<commit_message>
feat: implement live Google Sheets API sync with founder workspace
</commit_message>
<xml_diff>
--- a/docs/RevOps_Founder_Workspace_Planner.xlsx
+++ b/docs/RevOps_Founder_Workspace_Planner.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,6 +94,11 @@
       <color rgb="0016A34A"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -139,7 +144,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -161,11 +166,104 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -220,6 +318,18 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -605,7 +715,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -884,7 +993,7 @@
           <t>01.10.2026</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="22" t="inlineStr">
         <is>
           <t>✅ ВЫПОЛНЕНО</t>
         </is>
@@ -896,7 +1005,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>18% SQL, 18% слив, возврат 35%, 1-клик запуск на Desktop</t>
+          <t>Интерактивный B2B лендинг готов, протестирован, сохранен в Git</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1294,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
@@ -1200,10 +1308,26 @@
 Это УТП четко отделяет продукт от конкурентов. Мы не продаем софт — мы продаем результат: повышение эффективности отдела продаж.</t>
         </is>
       </c>
-    </row>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
+      <c r="B4" s="23" t="n"/>
+      <c r="C4" s="23" t="n"/>
+      <c r="D4" s="23" t="n"/>
+      <c r="E4" s="23" t="n"/>
+      <c r="F4" s="23" t="n"/>
+      <c r="G4" s="24" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="n"/>
+      <c r="G5" s="26" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="n"/>
+      <c r="B6" s="28" t="n"/>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+      <c r="E6" s="28" t="n"/>
+      <c r="F6" s="28" t="n"/>
+      <c r="G6" s="29" t="n"/>
+    </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
@@ -1249,11 +1373,14 @@
           <t>Руководитель видит, что план по выручке не выполняется, но причина скрыта в сотнях звонков (качество лидов? возражения? слив Next Step?). Наш продукт дает объективный математический ответ с точностью до рубля.</t>
         </is>
       </c>
+      <c r="D10" s="30" t="n"/>
+      <c r="E10" s="31" t="n"/>
       <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Отчет CFO + Экспресс-аудит 3 звонков</t>
         </is>
       </c>
+      <c r="G10" s="31" t="n"/>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
@@ -1271,11 +1398,14 @@
           <t>Руководитель тратит время на тренинги, но менеджеры продолжают отпускать клиентов фразой 'подумайте'. Наш продукт дает конкретные данные по 13 критериям для адресного коучинга каждого менеджера.</t>
         </is>
       </c>
+      <c r="D11" s="30" t="n"/>
+      <c r="E11" s="31" t="n"/>
       <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Пульт РОПа + Рейтинг менеджеров</t>
         </is>
       </c>
+      <c r="G11" s="31" t="n"/>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
@@ -1293,13 +1423,15 @@
           <t>Классический консалтинг занимает 2-3 месяца и стоит сотни тысяч. Наш продукт оцифровывает весь отдел за 7 дней пилотного спринта (29 000 ₽) с гарантией окупаемости.</t>
         </is>
       </c>
+      <c r="D12" s="30" t="n"/>
+      <c r="E12" s="31" t="n"/>
       <c r="F12" s="6" t="inlineStr">
         <is>
           <t>7-дневный пилотный спринт</t>
         </is>
       </c>
-    </row>
-    <row r="13"/>
+      <c r="G12" s="31" t="n"/>
+    </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
@@ -1318,11 +1450,15 @@
           <t>Слишком дорого (от 300 000 ₽) и долго (2-3 месяца). Дают PDF-отчет и уходят, внедрение виснет.</t>
         </is>
       </c>
+      <c r="C15" s="30" t="n"/>
+      <c r="D15" s="31" t="n"/>
       <c r="E15" s="18" t="inlineStr">
         <is>
           <t>RevOps OS: запуск за 7 дней, подписка от 49 000 ₽/мес, автоматический надзор 24/7.</t>
         </is>
       </c>
+      <c r="F15" s="30" t="n"/>
+      <c r="G15" s="31" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="17" t="inlineStr">
@@ -1335,11 +1471,15 @@
           <t>Слишком технично. Дают облако тегов и транскрипты, но не говорят РОПу, что делать и сколько денег теряется.</t>
         </is>
       </c>
+      <c r="C16" s="30" t="n"/>
+      <c r="D16" s="31" t="n"/>
       <c r="E16" s="18" t="inlineStr">
         <is>
           <t>RevOps OS: готовые алерты РОПу в Telegram и расчет потерь в рублях.</t>
         </is>
       </c>
+      <c r="F16" s="30" t="n"/>
+      <c r="G16" s="31" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
@@ -1352,11 +1492,15 @@
           <t>Заблокирован в РФ, не поддерживает amoCRM/Битрикс24, нарушает 152-ФЗ, стоит от $120/пользователь.</t>
         </is>
       </c>
+      <c r="C17" s="30" t="n"/>
+      <c r="D17" s="31" t="n"/>
       <c r="E17" s="18" t="inlineStr">
         <is>
           <t>RevOps OS: 100% серверы в РФ (152-ФЗ), нативная интеграция с amoCRM и Битрикс24.</t>
         </is>
       </c>
+      <c r="F17" s="30" t="n"/>
+      <c r="G17" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -1411,7 +1555,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1812,7 +1955,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2093,7 +2235,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
         <is>
@@ -2110,12 +2251,32 @@
 Удобно глянуть короткий One-Pager в Word на 1 страницу?</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="20" customHeight="1"/>
-    <row r="6" ht="20" customHeight="1"/>
-    <row r="7" ht="20" customHeight="1"/>
-    <row r="8" ht="20" customHeight="1"/>
-    <row r="9"/>
+      <c r="B4" s="23" t="n"/>
+      <c r="C4" s="23" t="n"/>
+      <c r="D4" s="23" t="n"/>
+      <c r="E4" s="23" t="n"/>
+      <c r="F4" s="24" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="25" t="n"/>
+      <c r="F5" s="26" t="n"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="25" t="n"/>
+      <c r="F6" s="26" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="25" t="n"/>
+      <c r="F7" s="26" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="27" t="n"/>
+      <c r="B8" s="28" t="n"/>
+      <c r="C8" s="28" t="n"/>
+      <c r="D8" s="28" t="n"/>
+      <c r="E8" s="28" t="n"/>
+      <c r="F8" s="29" t="n"/>
+    </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
@@ -2135,12 +2296,32 @@
 Удобно созвониться завтра в 11:30 на 10 минут?</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="20" customHeight="1"/>
-    <row r="13" ht="20" customHeight="1"/>
-    <row r="14" ht="20" customHeight="1"/>
-    <row r="15" ht="20" customHeight="1"/>
-    <row r="16"/>
+      <c r="B11" s="23" t="n"/>
+      <c r="C11" s="23" t="n"/>
+      <c r="D11" s="23" t="n"/>
+      <c r="E11" s="23" t="n"/>
+      <c r="F11" s="24" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="25" t="n"/>
+      <c r="F12" s="26" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="25" t="n"/>
+      <c r="F13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="25" t="n"/>
+      <c r="F14" s="26" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="27" t="n"/>
+      <c r="B15" s="28" t="n"/>
+      <c r="C15" s="28" t="n"/>
+      <c r="D15" s="28" t="n"/>
+      <c r="E15" s="28" t="n"/>
+      <c r="F15" s="29" t="n"/>
+    </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
@@ -2159,11 +2340,32 @@
 5. Оплата по безналичному расчету (Самозанятый, ст. 15 422-ФЗ, 0% НДС, чек 'Мой Налог').</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="20" customHeight="1"/>
-    <row r="20" ht="20" customHeight="1"/>
-    <row r="21" ht="20" customHeight="1"/>
-    <row r="22" ht="20" customHeight="1"/>
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="23" t="n"/>
+      <c r="D18" s="23" t="n"/>
+      <c r="E18" s="23" t="n"/>
+      <c r="F18" s="24" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="25" t="n"/>
+      <c r="F19" s="26" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="25" t="n"/>
+      <c r="F20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="25" t="n"/>
+      <c r="F21" s="26" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="27" t="n"/>
+      <c r="B22" s="28" t="n"/>
+      <c r="C22" s="28" t="n"/>
+      <c r="D22" s="28" t="n"/>
+      <c r="E22" s="28" t="n"/>
+      <c r="F22" s="29" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A4:F8"/>

</xml_diff>

<commit_message>
feat: add 📑 Инсайты_2_Исследований sheet to founder planner and live Google Sheets
</commit_message>
<xml_diff>
--- a/docs/RevOps_Founder_Workspace_Planner.xlsx
+++ b/docs/RevOps_Founder_Workspace_Planner.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎯 Спринты_и_Задачи" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💡 База_Знаний_и_УТП" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🤝 Пайплайн_Интеграторов" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎙️ Клиентские_Пилоты" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💬 Быстрые_Скрипты" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📑 Инсайты_2_Исследований" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🤝 Пайплайн_Интеграторов" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎙️ Клиентские_Пилоты" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💬 Быстрые_Скрипты" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -97,6 +98,12 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00B45309"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -263,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -330,6 +337,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1534,6 +1556,390 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Главные Тезисы и Инсайты 2-х Исследований Рынка РФ (43 стр. + 15 стр.) • Что нельзя упустить</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B3" s="32" t="inlineStr">
+        <is>
+          <t>Тема / Направление</t>
+        </is>
+      </c>
+      <c r="C3" s="32" t="inlineStr">
+        <is>
+          <t>Ключевой инсайт исследования (Тезис)</t>
+        </is>
+      </c>
+      <c r="D3" s="32" t="inlineStr">
+        <is>
+          <t>Почему это критически важно (Боль)</t>
+        </is>
+      </c>
+      <c r="E3" s="32" t="inlineStr">
+        <is>
+          <t>Решение в RevOps OS (Что делаем)</t>
+        </is>
+      </c>
+      <c r="F3" s="32" t="inlineStr">
+        <is>
+          <t>Золотое правило фаундера (Что нельзя упустить)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="54" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>Кризис B2B-продаж и рост CAC</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Стоимость привлечения лида (CAC) в РФ выросла в 2.5–4 раза. Яндекс Директ перегрет, холодные звонки дают &lt;1% конверсии.</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>Бизнес больше не может расти экстенсивно за счет вливания бюджета в рекламу. Слив каждого лида обходится в 2 000 – 15 000 ₽.</t>
+        </is>
+      </c>
+      <c r="E4" s="34" t="inlineStr">
+        <is>
+          <t>Фокус RevOps OS: не заливать новый трафик, а ликвидировать скрытые дыры в воронке, возвращая до 35% зависших сделок.</t>
+        </is>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>ГЛАВНЫЙ ПИТЧ: «Не тратьте еще 500к на рекламу — мы вернем вам от 1.5М ₽ из текущей базы лидов за 1-й месяц».</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="54" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B5" s="33" t="inlineStr">
+        <is>
+          <t>Уровень утечек 1: «Справочное бюро»</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>35% лидов сливаются на 1-м звонке: менеджеры подробно отвечают на вопросы клиента, но не берут инициативу и не закрывают на дату.</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Клиент получает бесплатную консультацию и уходит фразой «я подумаю». Менеджер ставит статус 'думает' и забывает.</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
+        <is>
+          <t>ИИ-Супервайзер по 13 критериям: жесткая проверка CR1 (Next Step). Если точная дата/время не названы — алерт РОПу через 15 минут.</t>
+        </is>
+      </c>
+      <c r="F5" s="35" t="inlineStr">
+        <is>
+          <t>ПРАВИЛО №1: Любой контакт без согласованной даты следующего звонка считается СЛИВOM сделки.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="54" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>Уровень утечек 2: «Слепота РОПа»</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>РОП слушает менее 2% звонков физически (при объеме 300–500 звонков в неделю). Выводы строятся на субъективных ощущениях.</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Тренинги по продажам не работают, потому что РОП не видит системных ошибок и не контролирует закрепление навыков.</t>
+        </is>
+      </c>
+      <c r="E6" s="34" t="inlineStr">
+        <is>
+          <t>Telegram-Шериф: 3 персонализированные сводки в день (08:30 утренний фокус, 14:00 SOS-алерты, 18:30 итог дня). Время РОПа: 15 мин/день.</t>
+        </is>
+      </c>
+      <c r="F6" s="35" t="inlineStr">
+        <is>
+          <t>ПРАВИЛО №2: РОПу не нужны графики на 100 страниц — ему нужен список из 3 конкретных сделок, которые горят прямо сейчас.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="B7" s="33" t="inlineStr">
+        <is>
+          <t>Уровень утечек 3: «Кладбище зомби-сделок»</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>В CRM висят миллионы на этапах «КП отправлено» или «В работе». При реальном аудите 65–75% из них брошены без касания 14+ дней.</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Отдел продаж создает иллюзию огромного пайплайна, а фактическая касса пуста. Собственник не видит реального прогноза выручки.</t>
+        </is>
+      </c>
+      <c r="E7" s="34" t="inlineStr">
+        <is>
+          <t>Автоматический Радар Выручки: маркировка зомби-сделок, расчет упущенной выгоды и выгрузка списка реанимации для дожима.</t>
+        </is>
+      </c>
+      <c r="F7" s="35" t="inlineStr">
+        <is>
+          <t>ПРАВИЛО №3: Реанимация 35% зависших сделок в первый месяц окупает подписку RevOps за 3 дня.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="B8" s="33" t="inlineStr">
+        <is>
+          <t>Позиционирование: RevOps-консультант</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>SaaS-платформы (MANGO, UIS) дают сырые транскрипты без действий. Классический консалтинг стоит от 300к ₽ и длится 2-3 месяца.</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Клиенту не нужен голый софт и не нужны длинные отчеты — ему нужны деньги в кассе и внедренные регламенты без затягивания.</t>
+        </is>
+      </c>
+      <c r="E8" s="34" t="inlineStr">
+        <is>
+          <t>Гибрид 'Софт + Консалтинг': 7-дневный пилотный спринт за 29 000 ₽ + регулярная супервизия с гарантией окупаемости.</t>
+        </is>
+      </c>
+      <c r="F8" s="35" t="inlineStr">
+        <is>
+          <t>ПРАВИЛО №4: «Мы не продаем софт. Мы находим, где вы теряете деньги, и пишем пошаговый план, как их вернуть».</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>Революция Unit-экономики STT</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Yandex SpeechKit Deferred (Batch STT) стоит ~0.02 ₽/мин ($0.0003), что в 3x дешевле Groq Whisper (~0.06 ₽/мин) и на 100% в РФ.</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Себестоимость распознавания всех звонков компании составляет всего 300–600 ₽ в месяц! Маржинальность нашего сервиса &gt; 90%.</t>
+        </is>
+      </c>
+      <c r="E9" s="36" t="inlineStr">
+        <is>
+          <t>Двухуровневая архитектура: Yandex Deferred для ночной 100% обработки звонков + Groq Whisper для быстрого (&lt;5 сек) экспресс-аудита.</t>
+        </is>
+      </c>
+      <c r="F9" s="35" t="inlineStr">
+        <is>
+          <t>ПРАВИЛО №5: Покупка своего сервера с RTX 4090 (~250к ₽) окупается только от 410 000 мин/мес. Облачный Yandex Deferred вне конкуренции.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>Лимиты API amoCRM и Битрикс24</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>amoCRM режет запросы при &gt; 7 rps. Облачный Битрикс24 жестко блокирует при &gt; 2 rps (пауза 0.5s). Вебхуки Битрикс24 лагают на 5-20 мин.</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Без встроенного рейт-лимитера и очереди выгрузка 500 звонков приводит к ошибкам 429/503 и полному падению синхронизации.</t>
+        </is>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>Внедрен RateLimiter (6 rps amo, 2 rps Б24), экспоненциальный бэкофф с джиттером и Batch API (до 50 операций в 1 запросе к Б24).</t>
+        </is>
+      </c>
+      <c r="F10" s="35" t="inlineStr">
+        <is>
+          <t>ПРАВИЛО №6: Строго выдерживать паузу не менее 0.51s между вызовами REST API Битрикс24 и группировать запросы в batch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>Защита от псевдодублей в CRM</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Клиенты звонят с разных номеров. Метод crm.duplicate.findbycomm в Битрикс24 возвращает максимум 20 записей. Менеджеры плодят дубли.</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Если прикрепить звонок к неверной закрытой сделке или старому дублю, РОП видит искаженную картину и теряет нить переговоров.</t>
+        </is>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>Алгоритм resolve_target_deal: нормализация номеров по E.164, приоритет открытых стадий воронки &gt; наибольшая сумма &gt; свежая дата.</t>
+        </is>
+      </c>
+      <c r="F11" s="35" t="inlineStr">
+        <is>
+          <t>ПРАВИЛО №7: Никогда не брать первую попавшуюся сделку из API. Всегда фильтровать по активности и сумме.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>Партнерство с интеграторами CRM</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Интеграторы amoCRM и Битрикс24 зарабатывают на разовой настройке и страдают от оттока. Им жизненно необходим recurring-доход.</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Интеграторы уже имеют доверие сотен лояльных B2B-клиентов. Партнерская сеть — главный бесплатный канал лидогенерации.</t>
+        </is>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>Оффер интеграторам: 25–30% пожизненного ревшара (от 12 250 до 36 000 ₽/мес на каждого клиента). Мы ведем 100% саппорта.</t>
+        </is>
+      </c>
+      <c r="F12" s="35" t="inlineStr">
+        <is>
+          <t>ПРАВИЛО №8: Интегратор не должен ничего внедрять сам. Он просто дает контакт клиента, а мы ежемесячно выплачиваем ему ревшар.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>Контур безопасности 152-ФЗ РФ</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Штрафы Роскомнадзора за нарушение 152-ФЗ и хранение ПДн за рубежом достигают 6–18 млн ₽. Любая СБ блокирует сервис без документов.</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Клиенты боятся проверок, а менеджеры могут пожаловаться в трудовую инспекцию на прослушку звонков.</t>
+        </is>
+      </c>
+      <c r="E13" s="36" t="inlineStr">
+        <is>
+          <t>Модуль PIISanitizer (токенизация телефонов/email) + комплект из 5 документов (согласие сотрудника, приказ, регламент 30 дней, чек НПД).</t>
+        </is>
+      </c>
+      <c r="F13" s="35" t="inlineStr">
+        <is>
+          <t>ПРАВИЛО №9: Юридический комплект снимает 100% страхов СБ и юристов клиента. Передавать его бесплатно при подключении пилота.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1927,7 +2333,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2211,7 +2617,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
style: calibrate row heights, column widths, text wrapping, and freeze panes across all sheets
</commit_message>
<xml_diff>
--- a/docs/RevOps_Founder_Workspace_Planner.xlsx
+++ b/docs/RevOps_Founder_Workspace_Planner.xlsx
@@ -270,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -350,6 +350,45 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -720,24 +759,25 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>RevOps Enterprise OS — Мастер-Планнер Спринтов и Задач Фаундера</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="26" customHeight="1">
+    <row r="2" ht="12" customHeight="1"/>
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>ID</t>
@@ -779,7 +819,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T-01</t>
@@ -790,7 +830,7 @@
           <t>CRM Connectors</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>Харденинг коннекторов amoCRM и Битрикс24 (защита от 429/503, батчинг, резолв дублей)</t>
         </is>
@@ -810,18 +850,18 @@
           <t>✅ ВЫПОЛНЕНО</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>amocrm_connector.py, bitrix24_connector.py</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>105 тестов проходят (100% PASS), лимиты 6 и 2 rps соблюдены</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>T-02</t>
@@ -832,7 +872,7 @@
           <t>Legal 152-ФЗ</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Сборка юридического комплекта безопасности для клиентов (5 шаблонов по 152-ФЗ)</t>
         </is>
@@ -852,18 +892,18 @@
           <t>✅ ВЫПОЛНЕНО</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>docs/152-ФЗ_Комплект_Безопасности.docx</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="16" t="inlineStr">
         <is>
           <t>Включает согласие менеджера, приказ, регламент 30 дней</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="34" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>T-03</t>
@@ -874,7 +914,7 @@
           <t>Partnerships</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>Оффер для интеграторов CRM с 25-30% ревшаром (One-Pager DOCX + скрипты TG/Email)</t>
         </is>
@@ -894,18 +934,18 @@
           <t>✅ ВЫПОЛНЕНО</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="16" t="inlineStr">
         <is>
           <t>docs/Партнерское_Предложение_Интеграторам_CRM.docx</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="16" t="inlineStr">
         <is>
           <t>Выплаты 12 250 - 36 000 ₽/мес на клиента, скрипты готовы</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1">
+    <row r="7" ht="34" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>T-04</t>
@@ -916,7 +956,7 @@
           <t>Speech Engine</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>Модуль распознавания речи speech_engine.py по 152-ФЗ с токенизацией ПДн</t>
         </is>
@@ -936,18 +976,18 @@
           <t>✅ ВЫПОЛНЕНО</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>speech_engine.py, test_speech_engine.py</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="16" t="inlineStr">
         <is>
           <t>Yandex SpeechKit Deferred (0.02 ₽/мин) + Groq fallback + Excel sync</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>T-05</t>
@@ -958,7 +998,7 @@
           <t>Lead Magnet</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>Экспресс-аудит 3 звонков (run_express_audit.py) для холодного/теплого выхода</t>
         </is>
@@ -978,18 +1018,18 @@
           <t>✅ ВЫПОЛНЕНО</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>run_express_audit.py, карточка HTML на Desktop</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>Выдает 1-page отчет + готовый текст в Telegram с расчетом потерь</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>T-06</t>
@@ -1000,7 +1040,7 @@
           <t>Web / Landing</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Интерактивный B2B-лендинг с калиброванным калькулятором ROI</t>
         </is>
@@ -1020,18 +1060,18 @@
           <t>✅ ВЫПОЛНЕНО</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>presentation/landing.html</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>Интерактивный B2B лендинг готов, протестирован, сохранен в Git</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
+    <row r="10" ht="34" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>T-07</t>
@@ -1042,7 +1082,7 @@
           <t>Product Demo</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Сборка 5-вкладочного Enterprise Showcase Excel (.xlsx) без скрытых формул</t>
         </is>
@@ -1062,18 +1102,18 @@
           <t>✅ ВЫПОЛНЕНО</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="16" t="inlineStr">
         <is>
           <t>RevOps_Platform_Demo_Sample.xlsx</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="16" t="inlineStr">
         <is>
           <t>Вшит в сайт через Base64 + лежит на Рабочем столе</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
+    <row r="11" ht="34" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>T-08</t>
@@ -1084,7 +1124,7 @@
           <t>GTM / Outreach</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>Первая рассылка оффера 10 интеграторам amoCRM и Битрикс24</t>
         </is>
@@ -1104,18 +1144,18 @@
           <t>⏳ В РАБОТЕ</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="16" t="inlineStr">
         <is>
           <t>Вкладка 'Пайплайн_Интеграторов'</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>Цель: 2 партнерских созвона на этой неделе</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1">
+    <row r="12" ht="34" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>T-09</t>
@@ -1126,7 +1166,7 @@
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>Развертывание веб-сайта на публичном домене / хостинге</t>
         </is>
@@ -1146,18 +1186,18 @@
           <t>⏳ В РАБОТЕ</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="16" t="inlineStr">
         <is>
           <t>example.qwen.site / Vercel</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="16" t="inlineStr">
         <is>
           <t>Код готов, проверить мобильную верстку и форму</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
+    <row r="13" ht="34" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>T-10</t>
@@ -1168,7 +1208,7 @@
           <t>Pilot Delivery</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>Проведение первого платного пилотного спринта (29 000 ₽)</t>
         </is>
@@ -1188,18 +1228,18 @@
           <t>📋 БЭКЛОГ</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="16" t="inlineStr">
         <is>
           <t>Пайплайн клиентов</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="16" t="inlineStr">
         <is>
           <t>Оцифровать 100% звонков первого клиента, выдать список спасения</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
+    <row r="14" ht="34" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>T-11</t>
@@ -1210,7 +1250,7 @@
           <t>Telegram Bot</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>Подключение вебхука живой CRM к telegram_bot.py для realtime-алертов</t>
         </is>
@@ -1230,18 +1270,18 @@
           <t>📋 БЭКЛОГ</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>telegram_bot.py</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>Утренний фокус в 08:30 + SOS-алерт при сливе Next Step</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
+    <row r="15" ht="34" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>T-12</t>
@@ -1252,7 +1292,7 @@
           <t>Legal NPD</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>Подготовка формы договора-оферты и акта для Самозанятого через 'Мой Налог'</t>
         </is>
@@ -1272,12 +1312,12 @@
           <t>📋 БЭКЛОГ</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>docs/Договор_Оферта_Самозанятый.docx</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>Статья 15 422-ФЗ, 0% НДС, безналичный расчет с юрлицами</t>
         </is>
@@ -1300,31 +1340,32 @@
   <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>База Знаний Продукта: Позиционирование, УТП и 3 Ключевые Боли Клиентов</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="2" ht="12" customHeight="1"/>
+    <row r="3" ht="26" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
         <is>
           <t>🔥 ГЛАВНОЕ УНИКАЛЬНОЕ ТОРГОВОЕ ПРЕДЛОЖЕНИЕ (УТП)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="4" ht="65" customHeight="1">
+      <c r="A4" s="37" t="inlineStr">
         <is>
           <t>«Мы не просто слушаем ваши звонки. Мы находим, почему вы теряете деньги, и пишем вам пошаговый план, как это исправить».
 Это УТП четко отделяет продукт от конкурентов. Мы не продаем софт — мы продаем результат: повышение эффективности отдела продаж.</t>
@@ -1350,131 +1391,133 @@
       <c r="F6" s="28" t="n"/>
       <c r="G6" s="29" t="n"/>
     </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+    <row r="7"/>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="38" t="inlineStr">
         <is>
           <t>🎯 3 КЛЮЧЕВЫЕ БОЛИ ЦЕЛЕВОЙ АУДИТОРИИ (Коммерческие директора, РОПы, Собственники)</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="39" t="inlineStr">
         <is>
           <t>Боль</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="39" t="inlineStr">
         <is>
           <t>Формулировка клиента</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="39" t="inlineStr">
         <is>
           <t>Суть проблемы в бизнесе</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="39" t="inlineStr">
         <is>
           <t>Наше решение в RevOps OS</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="40" t="inlineStr">
         <is>
           <t>Боль №1</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="41" t="inlineStr">
         <is>
           <t>«Я не знаю, почему мы теряем сделки»</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="42" t="inlineStr">
         <is>
           <t>Руководитель видит, что план по выручке не выполняется, но причина скрыта в сотнях звонков (качество лидов? возражения? слив Next Step?). Наш продукт дает объективный математический ответ с точностью до рубля.</t>
         </is>
       </c>
       <c r="D10" s="30" t="n"/>
       <c r="E10" s="31" t="n"/>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="43" t="inlineStr">
         <is>
           <t>Отчет CFO + Экспресс-аудит 3 звонков</t>
         </is>
       </c>
       <c r="G10" s="31" t="n"/>
     </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="40" t="inlineStr">
         <is>
           <t>Боль №2</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="41" t="inlineStr">
         <is>
           <t>«Мои менеджеры не растут»</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>Руководитель тратит время на тренинги, но менеджеры продолжают отпускать клиентов фразой 'подумайте'. Наш продукт дает конкретные данные по 13 критериям для адресного коучинга каждого менеджера.</t>
         </is>
       </c>
       <c r="D11" s="30" t="n"/>
       <c r="E11" s="31" t="n"/>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="43" t="inlineStr">
         <is>
           <t>Пульт РОПа + Рейтинг менеджеров</t>
         </is>
       </c>
       <c r="G11" s="31" t="n"/>
     </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="40" t="inlineStr">
         <is>
           <t>Боль №3</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="41" t="inlineStr">
         <is>
           <t>«Мне нужно быстро получить результат»</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C12" s="42" t="inlineStr">
         <is>
           <t>Классический консалтинг занимает 2-3 месяца и стоит сотни тысяч. Наш продукт оцифровывает весь отдел за 7 дней пилотного спринта (29 000 ₽) с гарантией окупаемости.</t>
         </is>
       </c>
       <c r="D12" s="30" t="n"/>
       <c r="E12" s="31" t="n"/>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="43" t="inlineStr">
         <is>
           <t>7-дневный пилотный спринт</t>
         </is>
       </c>
       <c r="G12" s="31" t="n"/>
     </row>
-    <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+    <row r="13"/>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="38" t="inlineStr">
         <is>
           <t>⚖️ МАТРИЦА ПОЗИЦИОНИРОВАНИЯ (ПОЧЕМУ МЫ ВЫИГРЫВАЕМ У КОНКУРЕНТОВ)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="44" t="inlineStr">
         <is>
           <t>Классический консалтинг</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="42" t="inlineStr">
         <is>
           <t>Слишком дорого (от 300 000 ₽) и долго (2-3 месяца). Дают PDF-отчет и уходят, внедрение виснет.</t>
         </is>
       </c>
       <c r="C15" s="30" t="n"/>
       <c r="D15" s="31" t="n"/>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E15" s="45" t="inlineStr">
         <is>
           <t>RevOps OS: запуск за 7 дней, подписка от 49 000 ₽/мес, автоматический надзор 24/7.</t>
         </is>
@@ -1482,20 +1525,20 @@
       <c r="F15" s="30" t="n"/>
       <c r="G15" s="31" t="n"/>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="44" t="inlineStr">
         <is>
           <t>Обычная речевая аналитика (SaaS)</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="42" t="inlineStr">
         <is>
           <t>Слишком технично. Дают облако тегов и транскрипты, но не говорят РОПу, что делать и сколько денег теряется.</t>
         </is>
       </c>
       <c r="C16" s="30" t="n"/>
       <c r="D16" s="31" t="n"/>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="45" t="inlineStr">
         <is>
           <t>RevOps OS: готовые алерты РОПу в Telegram и расчет потерь в рублях.</t>
         </is>
@@ -1503,20 +1546,20 @@
       <c r="F16" s="30" t="n"/>
       <c r="G16" s="31" t="n"/>
     </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="44" t="inlineStr">
         <is>
           <t>Зарубежный Revenue Intelligence (Gong)</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="42" t="inlineStr">
         <is>
           <t>Заблокирован в РФ, не поддерживает amoCRM/Битрикс24, нарушает 152-ФЗ, стоит от $120/пользователь.</t>
         </is>
       </c>
       <c r="C17" s="30" t="n"/>
       <c r="D17" s="31" t="n"/>
-      <c r="E17" s="18" t="inlineStr">
+      <c r="E17" s="45" t="inlineStr">
         <is>
           <t>RevOps OS: 100% серверы в РФ (152-ФЗ), нативная интеграция с amoCRM и Битрикс24.</t>
         </is>
@@ -1560,11 +1603,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -1574,6 +1617,7 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="12" customHeight="1"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="32" t="inlineStr">
         <is>
@@ -1606,321 +1650,321 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="54" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+    <row r="4" ht="68" customHeight="1">
+      <c r="A4" s="40" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="B4" s="33" t="inlineStr">
+      <c r="B4" s="44" t="inlineStr">
         <is>
           <t>Кризис B2B-продаж и рост CAC</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="42" t="inlineStr">
         <is>
           <t>Стоимость привлечения лида (CAC) в РФ выросла в 2.5–4 раза. Яндекс Директ перегрет, холодные звонки дают &lt;1% конверсии.</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="42" t="inlineStr">
         <is>
           <t>Бизнес больше не может расти экстенсивно за счет вливания бюджета в рекламу. Слив каждого лида обходится в 2 000 – 15 000 ₽.</t>
         </is>
       </c>
-      <c r="E4" s="34" t="inlineStr">
+      <c r="E4" s="46" t="inlineStr">
         <is>
           <t>Фокус RevOps OS: не заливать новый трафик, а ликвидировать скрытые дыры в воронке, возвращая до 35% зависших сделок.</t>
         </is>
       </c>
-      <c r="F4" s="35" t="inlineStr">
+      <c r="F4" s="47" t="inlineStr">
         <is>
           <t>ГЛАВНЫЙ ПИТЧ: «Не тратьте еще 500к на рекламу — мы вернем вам от 1.5М ₽ из текущей базы лидов за 1-й месяц».</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="54" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+    <row r="5" ht="68" customHeight="1">
+      <c r="A5" s="40" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="B5" s="33" t="inlineStr">
+      <c r="B5" s="44" t="inlineStr">
         <is>
           <t>Уровень утечек 1: «Справочное бюро»</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="42" t="inlineStr">
         <is>
           <t>35% лидов сливаются на 1-м звонке: менеджеры подробно отвечают на вопросы клиента, но не берут инициативу и не закрывают на дату.</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="42" t="inlineStr">
         <is>
           <t>Клиент получает бесплатную консультацию и уходит фразой «я подумаю». Менеджер ставит статус 'думает' и забывает.</t>
         </is>
       </c>
-      <c r="E5" s="34" t="inlineStr">
+      <c r="E5" s="46" t="inlineStr">
         <is>
           <t>ИИ-Супервайзер по 13 критериям: жесткая проверка CR1 (Next Step). Если точная дата/время не названы — алерт РОПу через 15 минут.</t>
         </is>
       </c>
-      <c r="F5" s="35" t="inlineStr">
+      <c r="F5" s="47" t="inlineStr">
         <is>
           <t>ПРАВИЛО №1: Любой контакт без согласованной даты следующего звонка считается СЛИВOM сделки.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+    <row r="6" ht="68" customHeight="1">
+      <c r="A6" s="40" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="B6" s="33" t="inlineStr">
+      <c r="B6" s="44" t="inlineStr">
         <is>
           <t>Уровень утечек 2: «Слепота РОПа»</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="42" t="inlineStr">
         <is>
           <t>РОП слушает менее 2% звонков физически (при объеме 300–500 звонков в неделю). Выводы строятся на субъективных ощущениях.</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="42" t="inlineStr">
         <is>
           <t>Тренинги по продажам не работают, потому что РОП не видит системных ошибок и не контролирует закрепление навыков.</t>
         </is>
       </c>
-      <c r="E6" s="34" t="inlineStr">
+      <c r="E6" s="46" t="inlineStr">
         <is>
           <t>Telegram-Шериф: 3 персонализированные сводки в день (08:30 утренний фокус, 14:00 SOS-алерты, 18:30 итог дня). Время РОПа: 15 мин/день.</t>
         </is>
       </c>
-      <c r="F6" s="35" t="inlineStr">
+      <c r="F6" s="47" t="inlineStr">
         <is>
           <t>ПРАВИЛО №2: РОПу не нужны графики на 100 страниц — ему нужен список из 3 конкретных сделок, которые горят прямо сейчас.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+    <row r="7" ht="68" customHeight="1">
+      <c r="A7" s="40" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="B7" s="33" t="inlineStr">
+      <c r="B7" s="44" t="inlineStr">
         <is>
           <t>Уровень утечек 3: «Кладбище зомби-сделок»</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C7" s="42" t="inlineStr">
         <is>
           <t>В CRM висят миллионы на этапах «КП отправлено» или «В работе». При реальном аудите 65–75% из них брошены без касания 14+ дней.</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="42" t="inlineStr">
         <is>
           <t>Отдел продаж создает иллюзию огромного пайплайна, а фактическая касса пуста. Собственник не видит реального прогноза выручки.</t>
         </is>
       </c>
-      <c r="E7" s="34" t="inlineStr">
+      <c r="E7" s="46" t="inlineStr">
         <is>
           <t>Автоматический Радар Выручки: маркировка зомби-сделок, расчет упущенной выгоды и выгрузка списка реанимации для дожима.</t>
         </is>
       </c>
-      <c r="F7" s="35" t="inlineStr">
+      <c r="F7" s="47" t="inlineStr">
         <is>
           <t>ПРАВИЛО №3: Реанимация 35% зависших сделок в первый месяц окупает подписку RevOps за 3 дня.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="54" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+    <row r="8" ht="68" customHeight="1">
+      <c r="A8" s="40" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="B8" s="33" t="inlineStr">
+      <c r="B8" s="44" t="inlineStr">
         <is>
           <t>Позиционирование: RevOps-консультант</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="42" t="inlineStr">
         <is>
           <t>SaaS-платформы (MANGO, UIS) дают сырые транскрипты без действий. Классический консалтинг стоит от 300к ₽ и длится 2-3 месяца.</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="42" t="inlineStr">
         <is>
           <t>Клиенту не нужен голый софт и не нужны длинные отчеты — ему нужны деньги в кассе и внедренные регламенты без затягивания.</t>
         </is>
       </c>
-      <c r="E8" s="34" t="inlineStr">
+      <c r="E8" s="46" t="inlineStr">
         <is>
           <t>Гибрид 'Софт + Консалтинг': 7-дневный пилотный спринт за 29 000 ₽ + регулярная супервизия с гарантией окупаемости.</t>
         </is>
       </c>
-      <c r="F8" s="35" t="inlineStr">
+      <c r="F8" s="47" t="inlineStr">
         <is>
           <t>ПРАВИЛО №4: «Мы не продаем софт. Мы находим, где вы теряете деньги, и пишем пошаговый план, как их вернуть».</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="54" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+    <row r="9" ht="68" customHeight="1">
+      <c r="A9" s="40" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="B9" s="33" t="inlineStr">
+      <c r="B9" s="44" t="inlineStr">
         <is>
           <t>Революция Unit-экономики STT</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="42" t="inlineStr">
         <is>
           <t>Yandex SpeechKit Deferred (Batch STT) стоит ~0.02 ₽/мин ($0.0003), что в 3x дешевле Groq Whisper (~0.06 ₽/мин) и на 100% в РФ.</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="42" t="inlineStr">
         <is>
           <t>Себестоимость распознавания всех звонков компании составляет всего 300–600 ₽ в месяц! Маржинальность нашего сервиса &gt; 90%.</t>
         </is>
       </c>
-      <c r="E9" s="36" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>Двухуровневая архитектура: Yandex Deferred для ночной 100% обработки звонков + Groq Whisper для быстрого (&lt;5 сек) экспресс-аудита.</t>
         </is>
       </c>
-      <c r="F9" s="35" t="inlineStr">
+      <c r="F9" s="47" t="inlineStr">
         <is>
           <t>ПРАВИЛО №5: Покупка своего сервера с RTX 4090 (~250к ₽) окупается только от 410 000 мин/мес. Облачный Yandex Deferred вне конкуренции.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="54" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+    <row r="10" ht="68" customHeight="1">
+      <c r="A10" s="40" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="B10" s="33" t="inlineStr">
+      <c r="B10" s="44" t="inlineStr">
         <is>
           <t>Лимиты API amoCRM и Битрикс24</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="42" t="inlineStr">
         <is>
           <t>amoCRM режет запросы при &gt; 7 rps. Облачный Битрикс24 жестко блокирует при &gt; 2 rps (пауза 0.5s). Вебхуки Битрикс24 лагают на 5-20 мин.</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="42" t="inlineStr">
         <is>
           <t>Без встроенного рейт-лимитера и очереди выгрузка 500 звонков приводит к ошибкам 429/503 и полному падению синхронизации.</t>
         </is>
       </c>
-      <c r="E10" s="36" t="inlineStr">
+      <c r="E10" s="48" t="inlineStr">
         <is>
           <t>Внедрен RateLimiter (6 rps amo, 2 rps Б24), экспоненциальный бэкофф с джиттером и Batch API (до 50 операций в 1 запросе к Б24).</t>
         </is>
       </c>
-      <c r="F10" s="35" t="inlineStr">
+      <c r="F10" s="47" t="inlineStr">
         <is>
           <t>ПРАВИЛО №6: Строго выдерживать паузу не менее 0.51s между вызовами REST API Битрикс24 и группировать запросы в batch.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="54" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+    <row r="11" ht="68" customHeight="1">
+      <c r="A11" s="40" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="B11" s="33" t="inlineStr">
+      <c r="B11" s="44" t="inlineStr">
         <is>
           <t>Защита от псевдодублей в CRM</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>Клиенты звонят с разных номеров. Метод crm.duplicate.findbycomm в Битрикс24 возвращает максимум 20 записей. Менеджеры плодят дубли.</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="42" t="inlineStr">
         <is>
           <t>Если прикрепить звонок к неверной закрытой сделке или старому дублю, РОП видит искаженную картину и теряет нить переговоров.</t>
         </is>
       </c>
-      <c r="E11" s="36" t="inlineStr">
+      <c r="E11" s="48" t="inlineStr">
         <is>
           <t>Алгоритм resolve_target_deal: нормализация номеров по E.164, приоритет открытых стадий воронки &gt; наибольшая сумма &gt; свежая дата.</t>
         </is>
       </c>
-      <c r="F11" s="35" t="inlineStr">
+      <c r="F11" s="47" t="inlineStr">
         <is>
           <t>ПРАВИЛО №7: Никогда не брать первую попавшуюся сделку из API. Всегда фильтровать по активности и сумме.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="54" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
+    <row r="12" ht="68" customHeight="1">
+      <c r="A12" s="40" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="B12" s="33" t="inlineStr">
+      <c r="B12" s="44" t="inlineStr">
         <is>
           <t>Партнерство с интеграторами CRM</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C12" s="42" t="inlineStr">
         <is>
           <t>Интеграторы amoCRM и Битрикс24 зарабатывают на разовой настройке и страдают от оттока. Им жизненно необходим recurring-доход.</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="42" t="inlineStr">
         <is>
           <t>Интеграторы уже имеют доверие сотен лояльных B2B-клиентов. Партнерская сеть — главный бесплатный канал лидогенерации.</t>
         </is>
       </c>
-      <c r="E12" s="36" t="inlineStr">
+      <c r="E12" s="48" t="inlineStr">
         <is>
           <t>Оффер интеграторам: 25–30% пожизненного ревшара (от 12 250 до 36 000 ₽/мес на каждого клиента). Мы ведем 100% саппорта.</t>
         </is>
       </c>
-      <c r="F12" s="35" t="inlineStr">
+      <c r="F12" s="47" t="inlineStr">
         <is>
           <t>ПРАВИЛО №8: Интегратор не должен ничего внедрять сам. Он просто дает контакт клиента, а мы ежемесячно выплачиваем ему ревшар.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="54" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
+    <row r="13" ht="68" customHeight="1">
+      <c r="A13" s="40" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="B13" s="33" t="inlineStr">
+      <c r="B13" s="44" t="inlineStr">
         <is>
           <t>Контур безопасности 152-ФЗ РФ</t>
         </is>
       </c>
-      <c r="C13" s="16" t="inlineStr">
+      <c r="C13" s="42" t="inlineStr">
         <is>
           <t>Штрафы Роскомнадзора за нарушение 152-ФЗ и хранение ПДн за рубежом достигают 6–18 млн ₽. Любая СБ блокирует сервис без документов.</t>
         </is>
       </c>
-      <c r="D13" s="16" t="inlineStr">
+      <c r="D13" s="42" t="inlineStr">
         <is>
           <t>Клиенты боятся проверок, а менеджеры могут пожаловаться в трудовую инспекцию на прослушку звонков.</t>
         </is>
       </c>
-      <c r="E13" s="36" t="inlineStr">
+      <c r="E13" s="48" t="inlineStr">
         <is>
           <t>Модуль PIISanitizer (токенизация телефонов/email) + комплект из 5 документов (согласие сотрудника, приказ, регламент 30 дней, чек НПД).</t>
         </is>
       </c>
-      <c r="F13" s="35" t="inlineStr">
+      <c r="F13" s="47" t="inlineStr">
         <is>
           <t>ПРАВИЛО №9: Юридический комплект снимает 100% страхов СБ и юристов клиента. Передавать его бесплатно при подключении пилота.</t>
         </is>
@@ -1943,25 +1987,26 @@
   <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Воронка Работы с Партнерами-Интеграторами CRM (Оффер 25–30% Recurring RevShare)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="26" customHeight="1">
+    <row r="2" ht="12" customHeight="1"/>
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>№</t>
@@ -2008,7 +2053,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4" ht="25" customHeight="1">
       <c r="A4" s="3" t="n">
         <v>1</v>
       </c>
@@ -2047,13 +2092,13 @@
           <t>15-20 активных</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="16" t="inlineStr">
         <is>
           <t>Отправить оффер в Telegram</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="25" customHeight="1">
       <c r="A5" s="3" t="n">
         <v>2</v>
       </c>
@@ -2092,13 +2137,13 @@
           <t>25-30 активных</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="16" t="inlineStr">
         <is>
           <t>Отправить One-Pager на почту</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="25" customHeight="1">
       <c r="A6" s="3" t="n">
         <v>3</v>
       </c>
@@ -2137,13 +2182,13 @@
           <t>10 активных</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" s="16" t="inlineStr">
         <is>
           <t>Созвон в Zoom на 15 минут</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
+    <row r="7" ht="25" customHeight="1">
       <c r="A7" s="19" t="n">
         <v>4</v>
       </c>
@@ -2154,9 +2199,9 @@
       <c r="F7" s="20" t="n"/>
       <c r="G7" s="20" t="n"/>
       <c r="H7" s="20" t="n"/>
-      <c r="I7" s="20" t="n"/>
-    </row>
-    <row r="8" ht="22" customHeight="1">
+      <c r="I7" s="49" t="n"/>
+    </row>
+    <row r="8" ht="25" customHeight="1">
       <c r="A8" s="19" t="n">
         <v>5</v>
       </c>
@@ -2167,9 +2212,9 @@
       <c r="F8" s="20" t="n"/>
       <c r="G8" s="20" t="n"/>
       <c r="H8" s="20" t="n"/>
-      <c r="I8" s="20" t="n"/>
-    </row>
-    <row r="9" ht="22" customHeight="1">
+      <c r="I8" s="49" t="n"/>
+    </row>
+    <row r="9" ht="25" customHeight="1">
       <c r="A9" s="19" t="n">
         <v>6</v>
       </c>
@@ -2180,9 +2225,9 @@
       <c r="F9" s="20" t="n"/>
       <c r="G9" s="20" t="n"/>
       <c r="H9" s="20" t="n"/>
-      <c r="I9" s="20" t="n"/>
-    </row>
-    <row r="10" ht="22" customHeight="1">
+      <c r="I9" s="49" t="n"/>
+    </row>
+    <row r="10" ht="25" customHeight="1">
       <c r="A10" s="19" t="n">
         <v>7</v>
       </c>
@@ -2193,9 +2238,9 @@
       <c r="F10" s="20" t="n"/>
       <c r="G10" s="20" t="n"/>
       <c r="H10" s="20" t="n"/>
-      <c r="I10" s="20" t="n"/>
-    </row>
-    <row r="11" ht="22" customHeight="1">
+      <c r="I10" s="49" t="n"/>
+    </row>
+    <row r="11" ht="25" customHeight="1">
       <c r="A11" s="19" t="n">
         <v>8</v>
       </c>
@@ -2206,9 +2251,9 @@
       <c r="F11" s="20" t="n"/>
       <c r="G11" s="20" t="n"/>
       <c r="H11" s="20" t="n"/>
-      <c r="I11" s="20" t="n"/>
-    </row>
-    <row r="12" ht="22" customHeight="1">
+      <c r="I11" s="49" t="n"/>
+    </row>
+    <row r="12" ht="25" customHeight="1">
       <c r="A12" s="19" t="n">
         <v>9</v>
       </c>
@@ -2219,9 +2264,9 @@
       <c r="F12" s="20" t="n"/>
       <c r="G12" s="20" t="n"/>
       <c r="H12" s="20" t="n"/>
-      <c r="I12" s="20" t="n"/>
-    </row>
-    <row r="13" ht="22" customHeight="1">
+      <c r="I12" s="49" t="n"/>
+    </row>
+    <row r="13" ht="25" customHeight="1">
       <c r="A13" s="19" t="n">
         <v>10</v>
       </c>
@@ -2232,9 +2277,9 @@
       <c r="F13" s="20" t="n"/>
       <c r="G13" s="20" t="n"/>
       <c r="H13" s="20" t="n"/>
-      <c r="I13" s="20" t="n"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
+      <c r="I13" s="49" t="n"/>
+    </row>
+    <row r="14" ht="25" customHeight="1">
       <c r="A14" s="19" t="n">
         <v>11</v>
       </c>
@@ -2245,9 +2290,9 @@
       <c r="F14" s="20" t="n"/>
       <c r="G14" s="20" t="n"/>
       <c r="H14" s="20" t="n"/>
-      <c r="I14" s="20" t="n"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
+      <c r="I14" s="49" t="n"/>
+    </row>
+    <row r="15" ht="25" customHeight="1">
       <c r="A15" s="19" t="n">
         <v>12</v>
       </c>
@@ -2258,9 +2303,9 @@
       <c r="F15" s="20" t="n"/>
       <c r="G15" s="20" t="n"/>
       <c r="H15" s="20" t="n"/>
-      <c r="I15" s="20" t="n"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
+      <c r="I15" s="49" t="n"/>
+    </row>
+    <row r="16" ht="25" customHeight="1">
       <c r="A16" s="19" t="n">
         <v>13</v>
       </c>
@@ -2271,9 +2316,9 @@
       <c r="F16" s="20" t="n"/>
       <c r="G16" s="20" t="n"/>
       <c r="H16" s="20" t="n"/>
-      <c r="I16" s="20" t="n"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
+      <c r="I16" s="49" t="n"/>
+    </row>
+    <row r="17" ht="25" customHeight="1">
       <c r="A17" s="19" t="n">
         <v>14</v>
       </c>
@@ -2284,9 +2329,9 @@
       <c r="F17" s="20" t="n"/>
       <c r="G17" s="20" t="n"/>
       <c r="H17" s="20" t="n"/>
-      <c r="I17" s="20" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
+      <c r="I17" s="49" t="n"/>
+    </row>
+    <row r="18" ht="25" customHeight="1">
       <c r="A18" s="19" t="n">
         <v>15</v>
       </c>
@@ -2297,9 +2342,9 @@
       <c r="F18" s="20" t="n"/>
       <c r="G18" s="20" t="n"/>
       <c r="H18" s="20" t="n"/>
-      <c r="I18" s="20" t="n"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
+      <c r="I18" s="49" t="n"/>
+    </row>
+    <row r="19" ht="25" customHeight="1">
       <c r="A19" s="19" t="n">
         <v>16</v>
       </c>
@@ -2310,9 +2355,9 @@
       <c r="F19" s="20" t="n"/>
       <c r="G19" s="20" t="n"/>
       <c r="H19" s="20" t="n"/>
-      <c r="I19" s="20" t="n"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
+      <c r="I19" s="49" t="n"/>
+    </row>
+    <row r="20" ht="25" customHeight="1">
       <c r="A20" s="19" t="n">
         <v>17</v>
       </c>
@@ -2323,7 +2368,7 @@
       <c r="F20" s="20" t="n"/>
       <c r="G20" s="20" t="n"/>
       <c r="H20" s="20" t="n"/>
-      <c r="I20" s="20" t="n"/>
+      <c r="I20" s="49" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2342,26 +2387,27 @@
   <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Воронка Клиентов: Экспресс-Аудит (0 ₽) → 7-дневный Пилот (29 000 ₽) → Подписка</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="26" customHeight="1">
+    <row r="2" ht="12" customHeight="1"/>
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>№</t>
@@ -2413,7 +2459,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4" ht="25" customHeight="1">
       <c r="A4" s="19" t="n">
         <v>1</v>
       </c>
@@ -2425,9 +2471,9 @@
       <c r="G4" s="20" t="n"/>
       <c r="H4" s="20" t="n"/>
       <c r="I4" s="20" t="n"/>
-      <c r="J4" s="20" t="n"/>
-    </row>
-    <row r="5" ht="24" customHeight="1">
+      <c r="J4" s="49" t="n"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
       <c r="A5" s="19" t="n">
         <v>2</v>
       </c>
@@ -2439,9 +2485,9 @@
       <c r="G5" s="20" t="n"/>
       <c r="H5" s="20" t="n"/>
       <c r="I5" s="20" t="n"/>
-      <c r="J5" s="20" t="n"/>
-    </row>
-    <row r="6" ht="24" customHeight="1">
+      <c r="J5" s="49" t="n"/>
+    </row>
+    <row r="6" ht="25" customHeight="1">
       <c r="A6" s="19" t="n">
         <v>3</v>
       </c>
@@ -2453,9 +2499,9 @@
       <c r="G6" s="20" t="n"/>
       <c r="H6" s="20" t="n"/>
       <c r="I6" s="20" t="n"/>
-      <c r="J6" s="20" t="n"/>
-    </row>
-    <row r="7" ht="24" customHeight="1">
+      <c r="J6" s="49" t="n"/>
+    </row>
+    <row r="7" ht="25" customHeight="1">
       <c r="A7" s="19" t="n">
         <v>4</v>
       </c>
@@ -2467,9 +2513,9 @@
       <c r="G7" s="20" t="n"/>
       <c r="H7" s="20" t="n"/>
       <c r="I7" s="20" t="n"/>
-      <c r="J7" s="20" t="n"/>
-    </row>
-    <row r="8" ht="24" customHeight="1">
+      <c r="J7" s="49" t="n"/>
+    </row>
+    <row r="8" ht="25" customHeight="1">
       <c r="A8" s="19" t="n">
         <v>5</v>
       </c>
@@ -2481,9 +2527,9 @@
       <c r="G8" s="20" t="n"/>
       <c r="H8" s="20" t="n"/>
       <c r="I8" s="20" t="n"/>
-      <c r="J8" s="20" t="n"/>
-    </row>
-    <row r="9" ht="24" customHeight="1">
+      <c r="J8" s="49" t="n"/>
+    </row>
+    <row r="9" ht="25" customHeight="1">
       <c r="A9" s="19" t="n">
         <v>6</v>
       </c>
@@ -2495,9 +2541,9 @@
       <c r="G9" s="20" t="n"/>
       <c r="H9" s="20" t="n"/>
       <c r="I9" s="20" t="n"/>
-      <c r="J9" s="20" t="n"/>
-    </row>
-    <row r="10" ht="24" customHeight="1">
+      <c r="J9" s="49" t="n"/>
+    </row>
+    <row r="10" ht="25" customHeight="1">
       <c r="A10" s="19" t="n">
         <v>7</v>
       </c>
@@ -2509,9 +2555,9 @@
       <c r="G10" s="20" t="n"/>
       <c r="H10" s="20" t="n"/>
       <c r="I10" s="20" t="n"/>
-      <c r="J10" s="20" t="n"/>
-    </row>
-    <row r="11" ht="24" customHeight="1">
+      <c r="J10" s="49" t="n"/>
+    </row>
+    <row r="11" ht="25" customHeight="1">
       <c r="A11" s="19" t="n">
         <v>8</v>
       </c>
@@ -2523,9 +2569,9 @@
       <c r="G11" s="20" t="n"/>
       <c r="H11" s="20" t="n"/>
       <c r="I11" s="20" t="n"/>
-      <c r="J11" s="20" t="n"/>
-    </row>
-    <row r="12" ht="24" customHeight="1">
+      <c r="J11" s="49" t="n"/>
+    </row>
+    <row r="12" ht="25" customHeight="1">
       <c r="A12" s="19" t="n">
         <v>9</v>
       </c>
@@ -2537,9 +2583,9 @@
       <c r="G12" s="20" t="n"/>
       <c r="H12" s="20" t="n"/>
       <c r="I12" s="20" t="n"/>
-      <c r="J12" s="20" t="n"/>
-    </row>
-    <row r="13" ht="24" customHeight="1">
+      <c r="J12" s="49" t="n"/>
+    </row>
+    <row r="13" ht="25" customHeight="1">
       <c r="A13" s="19" t="n">
         <v>10</v>
       </c>
@@ -2551,9 +2597,9 @@
       <c r="G13" s="20" t="n"/>
       <c r="H13" s="20" t="n"/>
       <c r="I13" s="20" t="n"/>
-      <c r="J13" s="20" t="n"/>
-    </row>
-    <row r="14" ht="24" customHeight="1">
+      <c r="J13" s="49" t="n"/>
+    </row>
+    <row r="14" ht="25" customHeight="1">
       <c r="A14" s="19" t="n">
         <v>11</v>
       </c>
@@ -2565,9 +2611,9 @@
       <c r="G14" s="20" t="n"/>
       <c r="H14" s="20" t="n"/>
       <c r="I14" s="20" t="n"/>
-      <c r="J14" s="20" t="n"/>
-    </row>
-    <row r="15" ht="24" customHeight="1">
+      <c r="J14" s="49" t="n"/>
+    </row>
+    <row r="15" ht="25" customHeight="1">
       <c r="A15" s="19" t="n">
         <v>12</v>
       </c>
@@ -2579,9 +2625,9 @@
       <c r="G15" s="20" t="n"/>
       <c r="H15" s="20" t="n"/>
       <c r="I15" s="20" t="n"/>
-      <c r="J15" s="20" t="n"/>
-    </row>
-    <row r="16" ht="24" customHeight="1">
+      <c r="J15" s="49" t="n"/>
+    </row>
+    <row r="16" ht="25" customHeight="1">
       <c r="A16" s="19" t="n">
         <v>13</v>
       </c>
@@ -2593,9 +2639,9 @@
       <c r="G16" s="20" t="n"/>
       <c r="H16" s="20" t="n"/>
       <c r="I16" s="20" t="n"/>
-      <c r="J16" s="20" t="n"/>
-    </row>
-    <row r="17" ht="24" customHeight="1">
+      <c r="J16" s="49" t="n"/>
+    </row>
+    <row r="17" ht="25" customHeight="1">
       <c r="A17" s="19" t="n">
         <v>14</v>
       </c>
@@ -2607,7 +2653,7 @@
       <c r="G17" s="20" t="n"/>
       <c r="H17" s="20" t="n"/>
       <c r="I17" s="20" t="n"/>
-      <c r="J17" s="20" t="n"/>
+      <c r="J17" s="49" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2626,29 +2672,29 @@
   <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Готовые Скрипты и Шаблоны Сообщений (Копировать / Вставить)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="26" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Шаблон 1: Telegram партнеру-интегратору CRM</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
+    <row r="4" ht="100" customHeight="1">
       <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Приветствую! Вижу, вы плотно занимаетесь внедрением amoCRM/Битрикс24.
@@ -2683,14 +2729,14 @@
       <c r="E8" s="28" t="n"/>
       <c r="F8" s="29" t="n"/>
     </row>
-    <row r="10" ht="24" customHeight="1">
+    <row r="10" ht="26" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Шаблон 2: Telegram собственнику после экспресс-аудита 3 звонков</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
+    <row r="11" ht="100" customHeight="1">
       <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Приветствую! Прогнали 3 ваших тестовых звонка через ИИ-супервизор RevOps.
@@ -2728,14 +2774,14 @@
       <c r="E15" s="28" t="n"/>
       <c r="F15" s="29" t="n"/>
     </row>
-    <row r="17" ht="24" customHeight="1">
+    <row r="17" ht="26" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Шаблон 3: Ответ юристу / службе безопасности по 152-ФЗ</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
+    <row r="18" ht="100" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
         <is>
           <t>Безопасность полностью закрыта по 152-ФЗ РФ:

</xml_diff>

<commit_message>
docs: sync task T-09 deployment status with live Qwen URL
</commit_message>
<xml_diff>
--- a/docs/RevOps_Founder_Workspace_Planner.xlsx
+++ b/docs/RevOps_Founder_Workspace_Planner.xlsx
@@ -1183,17 +1183,17 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>⏳ В РАБОТЕ</t>
+          <t>✅ ГОТОВО</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>example.qwen.site / Vercel</t>
+          <t>https://chat.qwen.ai/s/deploy/t_c34440cc-ed0a-44bd-b51c-8982f6336bcb</t>
         </is>
       </c>
       <c r="H12" s="16" t="inlineStr">
         <is>
-          <t>Код готов, проверить мобильную верстку и форму</t>
+          <t>Сайт развернут на Qwen Web Dev. Калькулятор, SheetJS Excel демо, TG @Reflecteddark и 152-ФЗ работают.</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,6 @@
       <c r="F6" s="28" t="n"/>
       <c r="G6" s="29" t="n"/>
     </row>
-    <row r="7"/>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="38" t="inlineStr">
         <is>
@@ -1496,7 +1495,6 @@
       </c>
       <c r="G12" s="31" t="n"/>
     </row>
-    <row r="13"/>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: update task T-09 with brand new custom domain ai-rop.ru
</commit_message>
<xml_diff>
--- a/docs/RevOps_Founder_Workspace_Planner.xlsx
+++ b/docs/RevOps_Founder_Workspace_Planner.xlsx
@@ -1188,12 +1188,12 @@
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>https://chat.qwen.ai/s/deploy/t_c34440cc-ed0a-44bd-b51c-8982f6336bcb</t>
+          <t>https://ai-rop.ru</t>
         </is>
       </c>
       <c r="H12" s="16" t="inlineStr">
         <is>
-          <t>Сайт развернут на Qwen Web Dev. Калькулятор, SheetJS Excel демо, TG @Reflecteddark и 152-ФЗ работают.</t>
+          <t>Собственный домен ai-rop.ru зарегистрирован на Reg.ru и подключен к GitHub Pages. 0 руб/мес за хостинг.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add 1-page Client Pilot Playbook docx and sync T-10 task
</commit_message>
<xml_diff>
--- a/docs/RevOps_Founder_Workspace_Planner.xlsx
+++ b/docs/RevOps_Founder_Workspace_Planner.xlsx
@@ -1225,17 +1225,17 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>📋 БЭКЛОГ</t>
+          <t>⏳ В РАБОТЕ</t>
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr">
         <is>
-          <t>Пайплайн клиентов</t>
+          <t>Боевой_Протокол_Клиент_За_7_Дней.docx</t>
         </is>
       </c>
       <c r="H13" s="16" t="inlineStr">
         <is>
-          <t>Оцифровать 100% звонков первого клиента, выдать список спасения</t>
+          <t>Сформирован 1-страничный протокол ведения клиента: Экспресс 0 ₽ -&gt; Пилот 29к -&gt; Ретейнер 79к</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sop): add first client protocol sheet and 20-min presentation script
</commit_message>
<xml_diff>
--- a/docs/RevOps_Founder_Workspace_Planner.xlsx
+++ b/docs/RevOps_Founder_Workspace_Planner.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🤝 Пайплайн_Интеграторов" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎙️ Клиентские_Пилоты" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💬 Быстрые_Скрипты" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🚀 Протокол_Первого_Клиента" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -106,8 +107,66 @@
       <color rgb="00B45309"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="0094A3B8"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00059669"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00334155"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="000F172A"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00E11D48"/>
+      <sz val="8.5"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -148,6 +207,36 @@
       <patternFill patternType="solid">
         <fgColor rgb="00EEF2FF"/>
         <bgColor rgb="00EEF2FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+        <bgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF1F2"/>
+        <bgColor rgb="00FFF1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -270,7 +359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -389,6 +478,75 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2828,4 +2986,830 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="50" t="inlineStr">
+        <is>
+          <t>🚀 RevOps Enterprise OS | Пошаговый Регламент Ведения Первого Клиента (End-to-End SOP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="51" t="inlineStr">
+        <is>
+          <t>Полная инструкция действий основателя: от входящей заявки до аудита 3 звонков за 24ч, закрытия пилота 45к-150к ₽ и абонентского сопровождения</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t>⚡ СКОРОСТЬ ПЕРВОГО ОТВЕТА</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="n"/>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>⏱️ ФОРМАТ ПЕРВОГО ДЕМО</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="n"/>
+      <c r="E4" s="53" t="inlineStr">
+        <is>
+          <t>🎯 ГЛАВНЫЙ ВХОДНОЙ ОФФЕР</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="n"/>
+      <c r="G4" s="54" t="inlineStr">
+        <is>
+          <t>💰 ЦЕЛЕВОЙ ЧЕК ПИЛОТА</t>
+        </is>
+      </c>
+      <c r="H4" s="20" t="n"/>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="55" t="inlineStr">
+        <is>
+          <t>&lt; 10 минут (в WhatsApp/TG)</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="n"/>
+      <c r="C5" s="55" t="inlineStr">
+        <is>
+          <t>Ровно 20 минут в Zoom</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="n"/>
+      <c r="E5" s="56" t="inlineStr">
+        <is>
+          <t>Тест 3 звонков за 24ч (0 ₽)</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="n"/>
+      <c r="G5" s="57" t="inlineStr">
+        <is>
+          <t>45 000 – 150 000 ₽</t>
+        </is>
+      </c>
+      <c r="H5" s="20" t="n"/>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="58" t="inlineStr">
+        <is>
+          <t>📋 ПОШАГОВЫЙ БОЕВОЙ АЛГОРИТМ: 12 ШАГОВ ВЕДЕНИЯ КЛИЕНТА</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="59" t="inlineStr">
+        <is>
+          <t>Шаг</t>
+        </is>
+      </c>
+      <c r="B8" s="59" t="inlineStr">
+        <is>
+          <t>Фаза воронки</t>
+        </is>
+      </c>
+      <c r="C8" s="59" t="inlineStr">
+        <is>
+          <t>Срок / Дедлайн</t>
+        </is>
+      </c>
+      <c r="D8" s="59" t="inlineStr">
+        <is>
+          <t>Что конкретно делает фаундер</t>
+        </is>
+      </c>
+      <c r="E8" s="59" t="inlineStr">
+        <is>
+          <t>Инструмент / Где лежит</t>
+        </is>
+      </c>
+      <c r="F8" s="59" t="inlineStr">
+        <is>
+          <t>Что сказать / Написать (скрипт)</t>
+        </is>
+      </c>
+      <c r="G8" s="59" t="inlineStr">
+        <is>
+          <t>Критерий успеха (DoD)</t>
+        </is>
+      </c>
+      <c r="H8" s="59" t="inlineStr">
+        <is>
+          <t>Опасная ошибка (Чего нельзя делать)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 1</t>
+        </is>
+      </c>
+      <c r="B9" s="60" t="inlineStr">
+        <is>
+          <t>Входящий лид</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>0 – 10 минут</t>
+        </is>
+      </c>
+      <c r="D9" s="62" t="inlineStr">
+        <is>
+          <t>Лид упал с сайта ai-rop.ru на почту info@ai-rop.ru или в Telegram @dm1918. Моментально пишем клиенту. Проводим экспресс-квалификацию по 3 вопросам.</t>
+        </is>
+      </c>
+      <c r="E9" s="62" t="inlineStr">
+        <is>
+          <t>Почта / Telegram @dm1918</t>
+        </is>
+      </c>
+      <c r="F9" s="63" t="inlineStr">
+        <is>
+          <t>«[Имя], добрый день! Получил вашу заявку на ai-rop.ru. Подскажите, сколько у вас менеджеров в отделе, какой средний чек и какую CRM используете?»</t>
+        </is>
+      </c>
+      <c r="G9" s="62" t="inlineStr">
+        <is>
+          <t>Получен ответ: подтверждено от 3 менеджеров и средний чек от 50 000 ₽.</t>
+        </is>
+      </c>
+      <c r="H9" s="64" t="inlineStr">
+        <is>
+          <t>Ждать больше 15 минут; отправлять громоздкие КП и коммерческие предложения в первом сообщении.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 2</t>
+        </is>
+      </c>
+      <c r="B10" s="65" t="inlineStr">
+        <is>
+          <t>Назначение демо</t>
+        </is>
+      </c>
+      <c r="C10" s="66" t="inlineStr">
+        <is>
+          <t>В течение 1 часа</t>
+        </is>
+      </c>
+      <c r="D10" s="67" t="inlineStr">
+        <is>
+          <t>Предложить 2 конкретных слота времени на выбор для 20-минутного Zoom-разбора. Скинуть ссылку на встречу и внести в календарь.</t>
+        </is>
+      </c>
+      <c r="E10" s="67" t="inlineStr">
+        <is>
+          <t>Google Календарь / Zoom / Яндекс.Телемост</t>
+        </is>
+      </c>
+      <c r="F10" s="68" t="inlineStr">
+        <is>
+          <t>«Отлично! Предлагаю созвониться на 20 минут в Zoom: покажу на пальцах, как ИИ слушает 100% звонков и находит потери. Завтра удобно в 11:30 или в 15:00?»</t>
+        </is>
+      </c>
+      <c r="G10" s="67" t="inlineStr">
+        <is>
+          <t>Встреча подтверждена клиентом и стоит в календаре.</t>
+        </is>
+      </c>
+      <c r="H10" s="64" t="inlineStr">
+        <is>
+          <t>Спрашивать: «Когда вам удобно?» — это размазывает договоренность.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 3</t>
+        </is>
+      </c>
+      <c r="B11" s="60" t="inlineStr">
+        <is>
+          <t>20-мин Презентация</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>День 2 (строго 20 мин)</t>
+        </is>
+      </c>
+      <c r="D11" s="62" t="inlineStr">
+        <is>
+          <t>Провести созвон строго по готовому Word-сценарию. Открыть сайт ai-rop.ru, Excel-калькулятор (3 числа) и Google Таблицу (13 стандартов B2B).</t>
+        </is>
+      </c>
+      <c r="E11" s="62" t="inlineStr">
+        <is>
+          <t>Сценарий_20_минутной_Презентации_RevOps.docx</t>
+        </is>
+      </c>
+      <c r="F11" s="63" t="inlineStr">
+        <is>
+          <t>Вести разговор по файлу: 3 мин боль -&gt; 4 мин Калькулятор потерь -&gt; 6 мин Живой аудит -&gt; 3 мин 152-ФЗ -&gt; 4 мин Оффер на тест 3 звонков.</t>
+        </is>
+      </c>
+      <c r="G11" s="62" t="inlineStr">
+        <is>
+          <t>Клиент в шоке от суммы потенциальных потерь и согласен на тест 3 звонков.</t>
+        </is>
+      </c>
+      <c r="H11" s="64" t="inlineStr">
+        <is>
+          <t>Пытаться продать годовой софт за 300к на первой встрече. Цель первой встречи — ТОЛЬКО получить 3 звонка!</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 4</t>
+        </is>
+      </c>
+      <c r="B12" s="65" t="inlineStr">
+        <is>
+          <t>Забор 3 звонков</t>
+        </is>
+      </c>
+      <c r="C12" s="66" t="inlineStr">
+        <is>
+          <t>Сразу после созвона</t>
+        </is>
+      </c>
+      <c r="D12" s="67" t="inlineStr">
+        <is>
+          <t>Отправить персональную ссылку на облачную папку для загрузки аудио (Яндекс.Диск/Google Drive) или предложить прислать файлы прямо в Telegram.</t>
+        </is>
+      </c>
+      <c r="E12" s="67" t="inlineStr">
+        <is>
+          <t>Яндекс.Диск / Telegram @dm1918</t>
+        </is>
+      </c>
+      <c r="F12" s="68" t="inlineStr">
+        <is>
+          <t>«[Имя], спасибо за созвон! Вот ссылка на закрытую папку: [Ссылка]. Загрузите 3 любых звонка за вчера (1 успешный и 2 слитых). Ровно через 24ч верну аудит».</t>
+        </is>
+      </c>
+      <c r="G12" s="67" t="inlineStr">
+        <is>
+          <t>3 аудиофайла (.mp3 или .wav) сохранены на вашем компьютере.</t>
+        </is>
+      </c>
+      <c r="H12" s="64" t="inlineStr">
+        <is>
+          <t>Давать сложные технические инструкции по API телефонии. Брать аудиофайлы простым архивом!</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 5</t>
+        </is>
+      </c>
+      <c r="B13" s="60" t="inlineStr">
+        <is>
+          <t>Защита 152-ФЗ</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>По запросу клиента</t>
+        </is>
+      </c>
+      <c r="D13" s="62" t="inlineStr">
+        <is>
+          <t>Если клиент или его СБ сомневаются в конфиденциальности — мгновенно отправить подписанный NDA и памятку по 152-ФЗ.</t>
+        </is>
+      </c>
+      <c r="E13" s="62" t="inlineStr">
+        <is>
+          <t>Папка «152 ФЗ» на Рабочем столе</t>
+        </is>
+      </c>
+      <c r="F13" s="63" t="inlineStr">
+        <is>
+          <t>«Мы работаем строго по 152-ФЗ РФ. Перед началом подписываем двусторонний NDA. Данные деперсонализируются в защищенном контуре. Направляю проект NDA».</t>
+        </is>
+      </c>
+      <c r="G13" s="62" t="inlineStr">
+        <is>
+          <t>NDA подписан с обеих сторон (скан или ЭДО).</t>
+        </is>
+      </c>
+      <c r="H13" s="64" t="inlineStr">
+        <is>
+          <t>Спорить со службой безопасности; говорить, что данные отправляются на зарубежные сервера.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 6</t>
+        </is>
+      </c>
+      <c r="B14" s="65" t="inlineStr">
+        <is>
+          <t>Fulfillment (Запуск ИИ)</t>
+        </is>
+      </c>
+      <c r="C14" s="66" t="inlineStr">
+        <is>
+          <t>В течение 4–6 часов</t>
+        </is>
+      </c>
+      <c r="D14" s="67" t="inlineStr">
+        <is>
+          <t>Запустить Start_Sales_Calls_AI.bat (Faster-Whisper на 8000, DeepSeek-R1 на 11434, n8n на 5678). Прогнать 3 аудиозаписи через транскрибацию и скоринг.</t>
+        </is>
+      </c>
+      <c r="E14" s="67" t="inlineStr">
+        <is>
+          <t>Start_Sales_Calls_AI.bat, transcriber_service</t>
+        </is>
+      </c>
+      <c r="F14" s="68" t="inlineStr">
+        <is>
+          <t>Автоматический процесс: получение расшифровки с тайм-кодами и скоринга по 13 критериям B2B.</t>
+        </is>
+      </c>
+      <c r="G14" s="67" t="inlineStr">
+        <is>
+          <t>Получены точные транскрипты и баллы соответствия по всем 13 стандартам.</t>
+        </is>
+      </c>
+      <c r="H14" s="64" t="inlineStr">
+        <is>
+          <t>Оставлять сырой нечитаемый текст без разбивки на реплики менеджера и клиента.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 7</t>
+        </is>
+      </c>
+      <c r="B15" s="60" t="inlineStr">
+        <is>
+          <t>Сборка клиентского отчета</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>В течение 8 часов</t>
+        </is>
+      </c>
+      <c r="D15" s="62" t="inlineStr">
+        <is>
+          <t>Сделать копию мастер-таблицы Google Sheets. Заполнить вкладку «ИИ_Аудит»: вставить цитаты, выставить зеленые/красные чипы, рассчитать недополученную маржу.</t>
+        </is>
+      </c>
+      <c r="E15" s="62" t="inlineStr">
+        <is>
+          <t>Google Sheets Master (gid 852624872)</t>
+        </is>
+      </c>
+      <c r="F15" s="63" t="inlineStr">
+        <is>
+          <t>Форматирование в корпоративном стиле: чипы ошибок, выделение желтым зон роста, формулы ROI.</t>
+        </is>
+      </c>
+      <c r="G15" s="62" t="inlineStr">
+        <is>
+          <t>Готовая брендированная ссылка на Google Таблицу с правами «Просмотр» для клиента.</t>
+        </is>
+      </c>
+      <c r="H15" s="64" t="inlineStr">
+        <is>
+          <t>Использовать неаккуратные шрифты или оставлять ошибки '###' в ячейках.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 8</t>
+        </is>
+      </c>
+      <c r="B16" s="65" t="inlineStr">
+        <is>
+          <t>Human-in-the-Loop</t>
+        </is>
+      </c>
+      <c r="C16" s="66" t="inlineStr">
+        <is>
+          <t>За 2 часа до сдачи</t>
+        </is>
+      </c>
+      <c r="D16" s="67" t="inlineStr">
+        <is>
+          <t>Фаундер лично переслушивает 2 ключевых спорных фрагмента. Формулирует 2 убийственных инсайта (например: 'Менеджер дал скидку 100к без торга').</t>
+        </is>
+      </c>
+      <c r="E16" s="67" t="inlineStr">
+        <is>
+          <t>Google Таблица + блокнот инсайтов</t>
+        </is>
+      </c>
+      <c r="F16" s="68" t="inlineStr">
+        <is>
+          <t>«Инсайт 1: Менеджер Александр не выявил ЛПР и отпустил клиента без даты повторного звонка. Инсайт 2: Слив скидки 15% снизил маржинальность сделки на 240 000 ₽».</t>
+        </is>
+      </c>
+      <c r="G16" s="67" t="inlineStr">
+        <is>
+          <t>Готовы 2 железобетонных факта потерь в деньгах, с которыми собственник не сможет поспорить.</t>
+        </is>
+      </c>
+      <c r="H16" s="64" t="inlineStr">
+        <is>
+          <t>Полагаться на 100% только на авто-генерацию ИИ без личной проверки спикером.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 9</t>
+        </is>
+      </c>
+      <c r="B17" s="60" t="inlineStr">
+        <is>
+          <t>Презентация аудита</t>
+        </is>
+      </c>
+      <c r="C17" s="61" t="inlineStr">
+        <is>
+          <t>Ровно через 24 часа</t>
+        </is>
+      </c>
+      <c r="D17" s="62" t="inlineStr">
+        <is>
+          <t>Созвон на 15 минут. Демонстрация экрана: «Вот ваши 3 звонка, вот где менеджеры слили 400 000 ₽». Показ готовой Google Таблицы.</t>
+        </is>
+      </c>
+      <c r="E17" s="62" t="inlineStr">
+        <is>
+          <t>Google Таблица клиента + Zoom</t>
+        </is>
+      </c>
+      <c r="F17" s="63" t="inlineStr">
+        <is>
+          <t>«[Имя], посмотрите строку 12: клиент спросил про рассрочку, менеджер ответил 'нет' и положил трубку. Здесь компания потеряла 350к. И это только 1 звонок из 3!»</t>
+        </is>
+      </c>
+      <c r="G17" s="62" t="inlineStr">
+        <is>
+          <t>Клиент признает: аудит объективен, проблема реальна и стоит больших денег.</t>
+        </is>
+      </c>
+      <c r="H17" s="64" t="inlineStr">
+        <is>
+          <t>Отправлять ссылку молча в мессенджер без личной демонстрации на созвоне.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 10</t>
+        </is>
+      </c>
+      <c r="B18" s="65" t="inlineStr">
+        <is>
+          <t>Закрытие на пилот</t>
+        </is>
+      </c>
+      <c r="C18" s="66" t="inlineStr">
+        <is>
+          <t>Финальные 5 мин созвона</t>
+        </is>
+      </c>
+      <c r="D18" s="67" t="inlineStr">
+        <is>
+          <t>Презентовать 7-дневный спринт: 100% звонков отдела за 45 000 – 75 000 ₽ (или спринт на месяц за 150 000 ₽) с гарантией окупаемости.</t>
+        </is>
+      </c>
+      <c r="E18" s="67" t="inlineStr">
+        <is>
+          <t>Спецификация пилота / Памятка 7 дней</t>
+        </is>
+      </c>
+      <c r="F18" s="68" t="inlineStr">
+        <is>
+          <t>«Мы отслушали 3 звонка и нашли слив на 400к. За 7 дней мы подключим 100% звонков отдела, дадим дашборд РОПу и спасем от 1 млн ₽. Стоимость пилота — 55 000 ₽. Стартуем?»</t>
+        </is>
+      </c>
+      <c r="G18" s="67" t="inlineStr">
+        <is>
+          <t>Устное «ДА» от собственника и запрос счета/договора.</t>
+        </is>
+      </c>
+      <c r="H18" s="64" t="inlineStr">
+        <is>
+          <t>Делать скидки при первом сомнении. Держать цену твердо, опираясь на ROI калькулятора.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 11</t>
+        </is>
+      </c>
+      <c r="B19" s="60" t="inlineStr">
+        <is>
+          <t>Оплата и договор</t>
+        </is>
+      </c>
+      <c r="C19" s="61" t="inlineStr">
+        <is>
+          <t>В течение 24 часов</t>
+        </is>
+      </c>
+      <c r="D19" s="62" t="inlineStr">
+        <is>
+          <t>Выставить счет от ИП/Самозанятого с QR-кодом. Направить типовой договор оказания услуг. Проконтролировать приход денег.</t>
+        </is>
+      </c>
+      <c r="E19" s="62" t="inlineStr">
+        <is>
+          <t>Банк-клиент (Точка / Тинькофф / Сбер)</t>
+        </is>
+      </c>
+      <c r="F19" s="63" t="inlineStr">
+        <is>
+          <t>«[Имя], направил договор и счет с QR-кодом на почту и в WhatsApp. Как только бухгалтерия проведет оплату, мы за 2 часа запускаем коннектор звонков».</t>
+        </is>
+      </c>
+      <c r="G19" s="62" t="inlineStr">
+        <is>
+          <t>Деньги поступили на расчетный счет. Подписан скан договора.</t>
+        </is>
+      </c>
+      <c r="H19" s="64" t="inlineStr">
+        <is>
+          <t>Начинать полноценную работу без предоплаты.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="52" t="inlineStr">
+        <is>
+          <t>Шаг 12</t>
+        </is>
+      </c>
+      <c r="B20" s="65" t="inlineStr">
+        <is>
+          <t>Сопровождение и LTV</t>
+        </is>
+      </c>
+      <c r="C20" s="66" t="inlineStr">
+        <is>
+          <t>Дни 1 – 7 пилота</t>
+        </is>
+      </c>
+      <c r="D20" s="67" t="inlineStr">
+        <is>
+          <t>Ежедневная выгрузка звонков, генерация утренней сводки в Telegram для РОПа в 09:00. В пятницу — итоговый отчет и продажа абонентской подписки (60к-120к/мес).</t>
+        </is>
+      </c>
+      <c r="E20" s="67" t="inlineStr">
+        <is>
+          <t>Telegram-бот @RevOps_Super_Audit_Bot</t>
+        </is>
+      </c>
+      <c r="F20" s="68" t="inlineStr">
+        <is>
+          <t>«За 7 дней мы разобрали 420 звонков, подняли показатель жесткого следующего шага с 32% до 78%, спасли 3 сделки на 1.2 млн ₽. Переходим на помесячный контракт?»</t>
+        </is>
+      </c>
+      <c r="G20" s="67" t="inlineStr">
+        <is>
+          <t>Подписан долгосрочный контракт на регулярную аналитику (MRR от 60 000 ₽).</t>
+        </is>
+      </c>
+      <c r="H20" s="64" t="inlineStr">
+        <is>
+          <t>Оставлять клиента без ежедневного контакта; не показывать динамику улучшений.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="58" t="inlineStr">
+        <is>
+          <t>💬 ШАБЛОНЫ БЫСТРЫХ СООБЩЕНИЙ ДЛЯ КОПИРОВАНИЯ (FAST COPY-PASTE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="69" t="inlineStr">
+        <is>
+          <t>Код</t>
+        </is>
+      </c>
+      <c r="B23" s="69" t="inlineStr">
+        <is>
+          <t>Событие</t>
+        </is>
+      </c>
+      <c r="C23" s="69" t="inlineStr">
+        <is>
+          <t>Канал</t>
+        </is>
+      </c>
+      <c r="D23" s="69" t="inlineStr">
+        <is>
+          <t>Готовый текст сообщения для клиента</t>
+        </is>
+      </c>
+      <c r="E23" s="30" t="n"/>
+      <c r="F23" s="30" t="n"/>
+      <c r="G23" s="30" t="n"/>
+      <c r="H23" s="31" t="n"/>
+    </row>
+    <row r="24" ht="42" customHeight="1">
+      <c r="A24" s="52" t="inlineStr">
+        <is>
+          <t>MSG-01</t>
+        </is>
+      </c>
+      <c r="B24" s="70" t="inlineStr">
+        <is>
+          <t>Первый ответ на заявку с сайта</t>
+        </is>
+      </c>
+      <c r="C24" s="71" t="inlineStr">
+        <is>
+          <t>Telegram / WhatsApp</t>
+        </is>
+      </c>
+      <c r="D24" s="72" t="inlineStr">
+        <is>
+          <t>«[Имя], приветствую! Получил вашу заявку на сервисе ai-rop.ru по аудиту звонков отдела продаж. Подскажите, пожалуйста: 1) Сколько менеджеров сейчас в линии? 2) Какой средний чек сделки? И какую CRM используете (amoCRM или Битрикс24)? Хочу подготовить релевантные примеры под вашу нишу перед созвоном».</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="n"/>
+      <c r="F24" s="20" t="n"/>
+      <c r="G24" s="20" t="n"/>
+      <c r="H24" s="20" t="n"/>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="52" t="inlineStr">
+        <is>
+          <t>MSG-02</t>
+        </is>
+      </c>
+      <c r="B25" s="70" t="inlineStr">
+        <is>
+          <t>Напоминание за 1 час до Zoom-демо</t>
+        </is>
+      </c>
+      <c r="C25" s="71" t="inlineStr">
+        <is>
+          <t>Telegram / WhatsApp</t>
+        </is>
+      </c>
+      <c r="D25" s="72" t="inlineStr">
+        <is>
+          <t>«[Имя], добрый день! Напоминаю, что через 1 час (в [Время]) у нас запланирован 20-минутный созвон в Zoom. Ссылка на встречу: [Ссылка]. Покажу на живых цифрах, как работает ИИ-аудит и сколько выручки теряется в звонках. До встречи!»</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="n"/>
+      <c r="F25" s="20" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="20" t="n"/>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="52" t="inlineStr">
+        <is>
+          <t>MSG-03</t>
+        </is>
+      </c>
+      <c r="B26" s="70" t="inlineStr">
+        <is>
+          <t>Инструкция по передаче 3 звонков</t>
+        </is>
+      </c>
+      <c r="C26" s="71" t="inlineStr">
+        <is>
+          <t>Telegram / WhatsApp</t>
+        </is>
+      </c>
+      <c r="D26" s="72" t="inlineStr">
+        <is>
+          <t>«[Имя], спасибо за встречу! Как договорились, жду от вас 3 любых аудиозаписи за вчера (один успешный звонок и два с сорвавшимися сделками). Загрузить можно сюда: [Ссылка на Яндекс.Диск] либо скинуть аудиофайлами прямо в этот чат. Завтра в [Время] верну готовую аналитику по 13 критериям».</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="n"/>
+      <c r="F26" s="20" t="n"/>
+      <c r="G26" s="20" t="n"/>
+      <c r="H26" s="20" t="n"/>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="52" t="inlineStr">
+        <is>
+          <t>MSG-04</t>
+        </is>
+      </c>
+      <c r="B27" s="70" t="inlineStr">
+        <is>
+          <t>Уведомление о готовности аудита</t>
+        </is>
+      </c>
+      <c r="C27" s="71" t="inlineStr">
+        <is>
+          <t>Telegram / WhatsApp</t>
+        </is>
+      </c>
+      <c r="D27" s="72" t="inlineStr">
+        <is>
+          <t>«[Имя], добрый день! Аудит ваших 3 звонков полностью готов. Нашли 2 критические системные ошибки менеджеров, из-за которых сорвались сделки на суммарно ~[Сумма] ₽. Собрал всё в персональную Google Таблицу. Предлагаю созвониться на 15 минут — выведу экран и покажу конкретные цитаты и точки слива. Удобно в [Время]?»</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="n"/>
+      <c r="F27" s="20" t="n"/>
+      <c r="G27" s="20" t="n"/>
+      <c r="H27" s="20" t="n"/>
+    </row>
+    <row r="28" ht="42" customHeight="1">
+      <c r="A28" s="52" t="inlineStr">
+        <is>
+          <t>MSG-05</t>
+        </is>
+      </c>
+      <c r="B28" s="70" t="inlineStr">
+        <is>
+          <t>Отправка счета на 7-дневный пилот</t>
+        </is>
+      </c>
+      <c r="C28" s="71" t="inlineStr">
+        <is>
+          <t>Email + Telegram</t>
+        </is>
+      </c>
+      <c r="D28" s="72" t="inlineStr">
+        <is>
+          <t>«[Имя], направил вам договор и счет на 7-дневный пилот RevOps (сумма 55 000 ₽). В стоимость входит анализ 100% звонков вашего отдела, ежедневная утренняя сводка РОПу в Telegram и оцифровка точек потерь. Оплатить можно по реквизитам или по QR-коду в счете. Стартуем сразу после подтверждения!»</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="n"/>
+      <c r="F28" s="20" t="n"/>
+      <c r="G28" s="20" t="n"/>
+      <c r="H28" s="20" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="C4:D4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(traffic): add Sprint 3 Telegram media plan, 20 channels, creatives, and UTM tracker to founder planner
</commit_message>
<xml_diff>
--- a/docs/RevOps_Founder_Workspace_Planner.xlsx
+++ b/docs/RevOps_Founder_Workspace_Planner.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💬 Быстрые_Скрипты" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔥 База_Лидов_HH" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🚀 Протокол_Первого_Клиента" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📢 Каналы_Продаж" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -142,8 +143,44 @@
       <color rgb="00E11D48"/>
       <sz val="8.5"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="007C3AED"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002563EB"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00059669"/>
+      <sz val="10.5"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -202,6 +239,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF1F2"/>
         <bgColor rgb="00FFF1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F3FF"/>
+        <bgColor rgb="00F5F3FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -324,7 +367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -465,6 +508,44 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5890,25 +5971,25 @@
           <t>⚡ СКОРОСТЬ ПЕРВОГО ОТВЕТА</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n"/>
+      <c r="B4" s="37" t="n"/>
       <c r="C4" s="10" t="inlineStr">
         <is>
           <t>⏱️ ФОРМАТ ПЕРВОГО ДЕМО</t>
         </is>
       </c>
-      <c r="D4" s="25" t="n"/>
+      <c r="D4" s="37" t="n"/>
       <c r="E4" s="6" t="inlineStr">
         <is>
           <t>🎯 ГЛАВНЫЙ ВХОДНОЙ ОФФЕР</t>
         </is>
       </c>
-      <c r="F4" s="25" t="n"/>
+      <c r="F4" s="37" t="n"/>
       <c r="G4" s="9" t="inlineStr">
         <is>
           <t>💰 ЦЕЛЕВОЙ ЧЕК ПИЛОТА</t>
         </is>
       </c>
-      <c r="H4" s="25" t="n"/>
+      <c r="H4" s="37" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="41" t="inlineStr">
@@ -5916,25 +5997,25 @@
           <t>&lt; 10 минут (в WhatsApp/TG)</t>
         </is>
       </c>
-      <c r="B5" s="25" t="n"/>
+      <c r="B5" s="37" t="n"/>
       <c r="C5" s="41" t="inlineStr">
         <is>
           <t>Ровно 20 минут в Zoom</t>
         </is>
       </c>
-      <c r="D5" s="25" t="n"/>
+      <c r="D5" s="37" t="n"/>
       <c r="E5" s="42" t="inlineStr">
         <is>
           <t>Тест 3 звонков за 24ч (0 ₽)</t>
         </is>
       </c>
-      <c r="F5" s="25" t="n"/>
+      <c r="F5" s="37" t="n"/>
       <c r="G5" s="43" t="inlineStr">
         <is>
           <t>45 000 – 150 000 ₽</t>
         </is>
       </c>
-      <c r="H5" s="25" t="n"/>
+      <c r="H5" s="37" t="n"/>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="44" t="inlineStr">
@@ -6543,10 +6624,10 @@
           <t>«[Имя], приветствую! Получил вашу заявку на сервисе ai-rop.ru по аудиту звонков отдела продаж. Подскажите, пожалуйста: 1) Сколько менеджеров сейчас в линии? 2) Какой средний чек сделки? И какую CRM используете (amoCRM или Битрикс24)? Хочу подготовить релевантные примеры под вашу нишу перед созвоном».</t>
         </is>
       </c>
-      <c r="E24" s="25" t="n"/>
-      <c r="F24" s="25" t="n"/>
-      <c r="G24" s="25" t="n"/>
-      <c r="H24" s="25" t="n"/>
+      <c r="E24" s="38" t="n"/>
+      <c r="F24" s="38" t="n"/>
+      <c r="G24" s="38" t="n"/>
+      <c r="H24" s="37" t="n"/>
     </row>
     <row r="25" ht="42" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -6569,10 +6650,10 @@
           <t>«[Имя], добрый день! Напоминаю, что через 1 час (в [Время]) у нас запланирован 20-минутный созвон в Zoom. Ссылка на встречу: [Ссылка]. Покажу на живых цифрах, как работает ИИ-аудит и сколько выручки теряется в звонках. До встречи!»</t>
         </is>
       </c>
-      <c r="E25" s="25" t="n"/>
-      <c r="F25" s="25" t="n"/>
-      <c r="G25" s="25" t="n"/>
-      <c r="H25" s="25" t="n"/>
+      <c r="E25" s="38" t="n"/>
+      <c r="F25" s="38" t="n"/>
+      <c r="G25" s="38" t="n"/>
+      <c r="H25" s="37" t="n"/>
     </row>
     <row r="26" ht="42" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
@@ -6595,10 +6676,10 @@
           <t>«[Имя], спасибо за встречу! Как договорились, жду от вас 3 любых аудиозаписи за вчера (один успешный звонок и два с сорвавшимися сделками). Загрузить можно сюда: [Ссылка на Яндекс.Диск] либо скинуть аудиофайлами прямо в этот чат. Завтра в [Время] верну готовую аналитику по 13 критериям».</t>
         </is>
       </c>
-      <c r="E26" s="25" t="n"/>
-      <c r="F26" s="25" t="n"/>
-      <c r="G26" s="25" t="n"/>
-      <c r="H26" s="25" t="n"/>
+      <c r="E26" s="38" t="n"/>
+      <c r="F26" s="38" t="n"/>
+      <c r="G26" s="38" t="n"/>
+      <c r="H26" s="37" t="n"/>
     </row>
     <row r="27" ht="42" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -6621,10 +6702,10 @@
           <t>«[Имя], добрый день! Аудит ваших 3 звонков полностью готов. Нашли 2 критические системные ошибки менеджеров, из-за которых сорвались сделки на суммарно ~[Сумма] ₽. Собрал всё в персональную Google Таблицу. Предлагаю созвониться на 15 минут — выведу экран и покажу конкретные цитаты и точки слива. Удобно в [Время]?»</t>
         </is>
       </c>
-      <c r="E27" s="25" t="n"/>
-      <c r="F27" s="25" t="n"/>
-      <c r="G27" s="25" t="n"/>
-      <c r="H27" s="25" t="n"/>
+      <c r="E27" s="38" t="n"/>
+      <c r="F27" s="38" t="n"/>
+      <c r="G27" s="38" t="n"/>
+      <c r="H27" s="37" t="n"/>
     </row>
     <row r="28" ht="42" customHeight="1">
       <c r="A28" s="10" t="inlineStr">
@@ -6647,10 +6728,10 @@
           <t>«[Имя], направил вам договор и счет на 7-дневный пилот RevOps (сумма 55 000 ₽). В стоимость входит анализ 100% звонков вашего отдела, ежедневная утренняя сводка РОПу в Telegram и оцифровка точек потерь. Оплатить можно по реквизитам или по QR-коду в счете. Стартуем сразу после подтверждения!»</t>
         </is>
       </c>
-      <c r="E28" s="25" t="n"/>
-      <c r="F28" s="25" t="n"/>
-      <c r="G28" s="25" t="n"/>
-      <c r="H28" s="25" t="n"/>
+      <c r="E28" s="38" t="n"/>
+      <c r="F28" s="38" t="n"/>
+      <c r="G28" s="38" t="n"/>
+      <c r="H28" s="37" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -6675,4 +6756,1374 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>📢 RevOps Enterprise OS | Медиаплан Платного Трафика в Telegram (B2B Sales &amp; CRM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>База отобранных Telegram-каналов для посевов, форматы 1/24 и 2/48, UTM-генератор, 3 готовых креатива и трекер окупаемости (ROI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="54" t="inlineStr">
+        <is>
+          <t>💰 БЮДЖЕТ ТЕСТА</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="n"/>
+      <c r="C4" s="55" t="inlineStr">
+        <is>
+          <t>👁️ ЦЕЛЕВОЙ ОХВАТ</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="n"/>
+      <c r="E4" s="54" t="inlineStr">
+        <is>
+          <t>🎯 КЛИКИ НА САЙТ (CTR ~2.5%)</t>
+        </is>
+      </c>
+      <c r="F4" s="25" t="n"/>
+      <c r="G4" s="56" t="inlineStr">
+        <is>
+          <t>📥 ЗАЯВКИ НА АУДИТ (0 ₽)</t>
+        </is>
+      </c>
+      <c r="H4" s="25" t="n"/>
+      <c r="I4" s="57" t="inlineStr">
+        <is>
+          <t>🚀 ЗАКРЫТЫЕ ПИЛОТЫ (ROI)</t>
+        </is>
+      </c>
+      <c r="J4" s="25" t="n"/>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="58" t="inlineStr">
+        <is>
+          <t>35 000 – 60 000 ₽</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="n"/>
+      <c r="C5" s="59" t="inlineStr">
+        <is>
+          <t>15 000 – 35 000 Views</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="n"/>
+      <c r="E5" s="60" t="inlineStr">
+        <is>
+          <t>450 – 850 кликов</t>
+        </is>
+      </c>
+      <c r="F5" s="25" t="n"/>
+      <c r="G5" s="61" t="inlineStr">
+        <is>
+          <t>25 – 45 заявок</t>
+        </is>
+      </c>
+      <c r="H5" s="25" t="n"/>
+      <c r="I5" s="62" t="inlineStr">
+        <is>
+          <t>3 – 6 сделок (165к-360к ₽)</t>
+        </is>
+      </c>
+      <c r="J5" s="25" t="n"/>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>🎯 РАЗДЕЛ 1: БАЗА 20 ОТОБРАННЫХ TELEGRAM-КАНАЛОВ ДЛЯ ЗАКУПА (B2B, CRM, РОПы, БИЗНЕС-РАЗБОРЫ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Код</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Категория</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Канал и Ссылка</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Целевая аудитория и специфика</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Формат</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Ориент. цена</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Креатив</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Персональная UTM-ссылка</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Статус контакта</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Переходы / Заявки</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>TG-01</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>B2B Продажи</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Заметки продавца B2B (@Salesnotes)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Сложные продажи, квалификация лидов, РОПы и КД</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>8 000 – 12 000 ₽</t>
+        </is>
+      </c>
+      <c r="G9" s="63" t="inlineStr">
+        <is>
+          <t>Пост 1 (CRM+Продажи)</t>
+        </is>
+      </c>
+      <c r="H9" s="64" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=salesnotes</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>TG-02</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>B2B Продажи</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>План продаж — М. Графский (@grafsky_b2b)</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Системные руководители ОП, регламенты и скрипты</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>1/24</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>10 000 – 15 000 ₽</t>
+        </is>
+      </c>
+      <c r="G10" s="63" t="inlineStr">
+        <is>
+          <t>Пост 2 (Кейс 340к)</t>
+        </is>
+      </c>
+      <c r="H10" s="65" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=grafsky_b2b</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>TG-03</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>B2B Продажи</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Продажник +1 (@floor_99)</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Практические кейсы, холодные звонки, дожим сделок</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>6 000 – 9 000 ₽</t>
+        </is>
+      </c>
+      <c r="G11" s="63" t="inlineStr">
+        <is>
+          <t>Пост 1 (CRM+Продажи)</t>
+        </is>
+      </c>
+      <c r="H11" s="64" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=floor_99</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>TG-04</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>B2B Продажи</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Ерохин про B2B продажи (@yerokhin_b2b)</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Топ-менеджмент B2B с длинными циклами и чеками</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>12 000 – 18 000 ₽</t>
+        </is>
+      </c>
+      <c r="G12" s="63" t="inlineStr">
+        <is>
+          <t>Пост 2 (Кейс 340к)</t>
+        </is>
+      </c>
+      <c r="H12" s="65" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=yerokhin_b2b</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>TG-05</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>B2B Продажи</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Охотники за продажами (@avsoln)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>А. Солнцева: разборы скриптов, возражение 'дорого'</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>1/24</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>7 000 – 10 000 ₽</t>
+        </is>
+      </c>
+      <c r="G13" s="63" t="inlineStr">
+        <is>
+          <t>Пост 1 (CRM+Продажи)</t>
+        </is>
+      </c>
+      <c r="H13" s="64" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=avsoln</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>TG-06</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>CRM / Интеграторы</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>50 оттенков CRM (@crm50)</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Юрий Николаев (Битрикс24), фанаты автоматизации ОП</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Натив / 2/48</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>12 000 – 18 000 ₽</t>
+        </is>
+      </c>
+      <c r="G14" s="63" t="inlineStr">
+        <is>
+          <t>Пост 1 (CRM+Продажи)</t>
+        </is>
+      </c>
+      <c r="H14" s="65" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=crm50</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>TG-07</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>CRM / Интеграторы</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Блог RocketSales (@rocketsales_blog)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Крупнейший интегратор amoCRM, активный B2B</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>8 000 – 14 000 ₽</t>
+        </is>
+      </c>
+      <c r="G15" s="63" t="inlineStr">
+        <is>
+          <t>Пост 3 (Атака на минуты)</t>
+        </is>
+      </c>
+      <c r="H15" s="64" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=rocketsales</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>TG-08</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>CRM / Интеграторы</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>ИНТРОvert | CRM (@introvert_crm)</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Внедрение сложных IT-решений поверх amoCRM</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>9 000 – 15 000 ₽</t>
+        </is>
+      </c>
+      <c r="G16" s="63" t="inlineStr">
+        <is>
+          <t>Пост 3 (Атака на минуты)</t>
+        </is>
+      </c>
+      <c r="H16" s="65" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=introvert</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>TG-09</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>CRM / Интеграторы</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Секреты Битрикс24 и amoCRM (@crm_secrets)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>РОПы и предприниматели в поиске ИИ-виджетов</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>5 000 – 8 000 ₽</t>
+        </is>
+      </c>
+      <c r="G17" s="63" t="inlineStr">
+        <is>
+          <t>Пост 1 (CRM+Продажи)</t>
+        </is>
+      </c>
+      <c r="H17" s="64" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=crm_secrets</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>TG-10</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>CRM / Маркетинг</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Комплето B2B (@completo_ru)</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>B2B Sales Performance: маркетинг + CRM + продажи</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>15 000 – 22 000 ₽</t>
+        </is>
+      </c>
+      <c r="G18" s="63" t="inlineStr">
+        <is>
+          <t>Пост 1 (CRM+Продажи)</t>
+        </is>
+      </c>
+      <c r="H18" s="65" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=completo</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>TG-11</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>CRM / Лидген</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Андрей Шишкин про B2B лидген (@andrew_shishkin)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Автоматизация воронки, экономия времени РОПа</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>1/24</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>6 000 – 9 000 ₽</t>
+        </is>
+      </c>
+      <c r="G19" s="63" t="inlineStr">
+        <is>
+          <t>Пост 2 (Кейс 340к)</t>
+        </is>
+      </c>
+      <c r="H19" s="64" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=andrew_shishkin</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>TG-12</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>CRM / Аналитика</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>B2B-медиа | Продажи (@b2bmedia)</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Исследования воронки, конверсии коммерческих служб</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>7 000 – 11 000 ₽</t>
+        </is>
+      </c>
+      <c r="G20" s="63" t="inlineStr">
+        <is>
+          <t>Пост 1 (CRM+Продажи)</t>
+        </is>
+      </c>
+      <c r="H20" s="65" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=b2bmedia</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>TG-13</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Бизнес-Разборы</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Resulting | Отделы продаж (@resulting_ru)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Агентство М. Гребенюка: 100% концентрация РОПов</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>По запросу</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>50 000 – 90 000 ₽</t>
+        </is>
+      </c>
+      <c r="G21" s="63" t="inlineStr">
+        <is>
+          <t>Пост 2 (Кейс 340к)</t>
+        </is>
+      </c>
+      <c r="H21" s="64" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=resulting</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>TG-14</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Бизнес-Разборы</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Бизнес-Разборы | Кейсы (@biz_razbory)</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Ошибки управления, сливы лидов в реалити-шоу</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>10 000 – 16 000 ₽</t>
+        </is>
+      </c>
+      <c r="G22" s="63" t="inlineStr">
+        <is>
+          <t>Пост 2 (Кейс 340к)</t>
+        </is>
+      </c>
+      <c r="H22" s="65" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=biz_razbory</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>TG-15</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Системный Бизнес</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Дневник Предпринимателя (@vysotsky_consulting)</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Александр Высоцкий: выход из операционки</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>1/24</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>25 000 – 45 000 ₽</t>
+        </is>
+      </c>
+      <c r="G23" s="63" t="inlineStr">
+        <is>
+          <t>Пост 1 (CRM+Продажи)</t>
+        </is>
+      </c>
+      <c r="H23" s="64" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=vysotsky</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>TG-16</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>Системный Бизнес</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Oy-li | Екатерина Уколова (@oyli_ru)</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Чек-листы, регламенты ОП, жесткая CRM-аналитика</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>30 000 – 50 000 ₽</t>
+        </is>
+      </c>
+      <c r="G24" s="63" t="inlineStr">
+        <is>
+          <t>Пост 1 (CRM+Продажи)</t>
+        </is>
+      </c>
+      <c r="H24" s="65" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=oyli</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>TG-17</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Менеджмент B2B</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Максим Батырев | Комбат (@batyrev_maxim)</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Армия российских РОПов и коммерческих директоров</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>1/24</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>40 000 – 70 000 ₽</t>
+        </is>
+      </c>
+      <c r="G25" s="63" t="inlineStr">
+        <is>
+          <t>Пост 2 (Кейс 340к)</t>
+        </is>
+      </c>
+      <c r="H25" s="64" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=batyrev</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>TG-18</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>ИИ в Продажах</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Сергей Кошечкин | Продажи (@koshechkin_sales)</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Жесткий практик, автоматизация и ИИ в коммерции</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>8 000 – 14 000 ₽</t>
+        </is>
+      </c>
+      <c r="G26" s="63" t="inlineStr">
+        <is>
+          <t>Пост 1 (CRM+Продажи)</t>
+        </is>
+      </c>
+      <c r="H26" s="65" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=koshechkin</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>TG-19</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Тяжелый B2B</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>MANAGED / Иван Чирков (@managed_ru)</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Операционная эффективность, оцифровка процессов</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>9 000 – 14 000 ₽</t>
+        </is>
+      </c>
+      <c r="G27" s="63" t="inlineStr">
+        <is>
+          <t>Пост 1 (CRM+Продажи)</t>
+        </is>
+      </c>
+      <c r="H27" s="64" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=managed</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>TG-20</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>ИИ в Бизнесе</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>ИИ в бизнесе | Нейросети (@ai_business_ru)</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Практика внедрения нейросетей в коммерческие отделы</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>2/48</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>5 000 – 8 000 ₽</t>
+        </is>
+      </c>
+      <c r="G28" s="63" t="inlineStr">
+        <is>
+          <t>Пост 3 (Атака на минуты)</t>
+        </is>
+      </c>
+      <c r="H28" s="65" t="inlineStr">
+        <is>
+          <t>https://ai-rop.ru/?utm_source=tg&amp;utm_medium=ai_business</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>В плане на контакт</t>
+        </is>
+      </c>
+      <c r="J28" s="8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="66" t="inlineStr">
+        <is>
+          <t>📝 РАЗДЕЛ 2: ГОТОВЫЕ РЕКЛАМНЫЕ ПОСТЫ ДЛЯ ЗАКАЗА В TELEGRAM (FAST COPY-PASTE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="67" t="inlineStr">
+        <is>
+          <t>📌 Пост 1 (Комбо: Продажи + CRM) | Для каналов: @crm50, @completo_ru, @Salesnotes, @crm_secrets, @introvert_crm</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="110" customHeight="1">
+      <c r="A32" s="31" t="inlineStr">
+        <is>
+          <t>Почему ваша CRM показывает прибыль, которой на самом деле нет? 📉
+Вы внедрили amoCRM или Битрикс24, настроили роботов, но менеджеры всё равно забивают на стандарты:
+• Отправляют КП на «кладбище почты» без фиксации даты следующего шага.
+• Сдаются при первом же возражении «Дорого» и сливают чек.
+• Пишут в комментариях абстрактное «клиент думает», маскируя уходящий лид.
+РОП физически успевает отслушать лишь 2–3% звонков, а остальные 98% воронки остаются в слепой зоне.
+Платформа RevOps OS PRO объединяет речевую аналитику ИИ и вашу CRM, полностью ликвидируя сливы:
+🟢 ИИ слушает 100% звонков: Нейросеть Whisper Pro расшифровывает каждый разговор и оценивает его по 13 жестким бизнес-критериям.
+🟢 Мгновенные алерты в Telegram: Если менеджер грубит, называет неверную цену или отпускает клиента — РОП получает уведомление со сценарием спасения сделки за 30 секунд.
+🟢 Автозаполнение карточек: ИИ сам пишет краткое резюме (Executive Summary) и выставляет договоренности прямо в CRM. Менеджеры больше не тратят время на рутину.
+Результат: Внедрение за 15 минут по API без остановки отдела. Спасение даже одной крупной сделки полностью окупает годовую подписку.
+Перестаньте гадать, сколько денег пролетает мимо кассы. Загрузите 3 вчерашних звонка ваших менеджеров — ИИ бесплатно оцифрует сумму денежного риска в рублях за 20 минут.
+👉 [Получить экспресс-аудит 3 звонков (0 ₽)] {ССЫЛКА_С_UTM}</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="67" t="inlineStr">
+        <is>
+          <t>📌 Пост 2 (Кейс-разбор в стиле шоу Гребенюка) | Для каналов: @resulting_ru, @biz_razbory, @floor_99, @batyrev_maxim, @grafsky_b2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="110" customHeight="1">
+      <c r="A34" s="31" t="inlineStr">
+        <is>
+          <t>«Ну ладно... Я просто скину вам КП на почту». Как менеджер своими руками похоронил сделку на 340 000 ₽. Пошаговый разбор 🔥
+Знакомая фраза? Руководитель думает, что отдел продаж работает, а ИИ-супервайзер RevOps OS видит реальность:
+1. Менеджер 40 минут рассказывал о продукте секретарю, так и не узнав, кто принимает финансовое решение (ЛПР).
+2. Услышав дежурное «Отправьте предложение, мы посмотрим», покорно согласился и положил трубку.
+3. Не назначил точную дату и время звонка. Сделка ушла на кладбище забытых лидов.
+Убыток компании: 340 000 ₽ чистой маржи + 6 500 ₽ сгоревшего бюджета Яндекс.Директа.
+РОП этого звонка не слышал, потому что физически успевает разобрать не более 5 диалогов в неделю.
+Платформа RevOps OS слушает 100% звонков менеджеров за секунды:
+• Находит фатальные ошибки по 13 критериям B2B.
+• Присылает РОПу алерт в Telegram за 30 секунд со сценарием: что сказать клиенту, чтобы вернуть его в сделку.
+• Показывает сумму упущенной прибыли прямо в рублях.
+Хотите узнать, где прямо сейчас сливают ваши менеджеры? Отправьте 3 вчерашних звонка — ИИ разберет их бесплатно за 20 минут.
+👉 [Проверить 3 звонка отдела продаж (0 ₽)] {ССЫЛКА_С_UTM}</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="67" t="inlineStr">
+        <is>
+          <t>📌 Пост 3 (Переманивание клиентов с imot.io и Mango) | Для каналов: @rocketsales_blog, @introvert_crm, @ai_business_ru, @crm50</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="110" customHeight="1">
+      <c r="A36" s="31" t="inlineStr">
+        <is>
+          <t>Платите за минуты речевой аналитики? Хватит считать секунды разговоров ваших менеджеров! ⏱️
+Классические системы аналитики продают «пакеты минут»: 50 000 ₽ за 10 000 минут. Если в отделе 8–10 менеджеров, лимит сгорает за 2 недели, а дальше вам выставляют счета на 120к–190к рублей.
+При этом вы получаете гору сложных графиков и облако тегов, в которых РОП всё равно не понимает, кому звонить.
+Переходите на RevOps OS Pro:
+✅ Фиксированная цена за команду без подсчета минут: контролируйте 100% разговоров без страха переплаты.
+✅ Деньги вместо графиков: ИИ показывает не «длительность пауз», а сумму в рублях, которую менеджер поставил под угрозу срыва.
+✅ Перенос настроек за 1 рабочий день: перенесем ваши словари и регламенты без стресса для IT-отдела.
+🎁 Спец-оффер при переходе: 1 месяц аналитики в подарок при переезде с поминутных тарифов.
+👉 [Узнать условия переезда и получить тест 3 звонков] {ССЫЛКА_С_UTM}</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>🛡️ РАЗДЕЛ 3: ПРАВИЛА ЗАКУПА В TELEGRAM (КАК СБИТЬ ЦЕНУ И НЕ СЛИТЬ БЮДЖЕТ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>Правило 1: Проверка через TGStat</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>Перед оплатой обязательно вбейте канал на tgstat.ru. Смотрите на ER (вовлеченность должна быть &gt;15-20%) и график суточного охвата: если посты читают равномерно, а не скачком в 03:00 ночи — накрутки ботами нет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>Правило 2: Формат размещения 2/48</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>Не берите 1/24 (быстро смоется лентой). Для длинных экспертных постов B2B просите формат 2/48 (2 часа в топе без перекрытия другими постами и 48 часов в ленте), либо формат 'без удаления'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>Правило 3: Скрипт торга со скидкой 10-20%</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>Пишите админу прямо: «Тестируем новый ИИ-сервис для B2B отделов продаж. Если отдача будет хорошей — зайдем на постоянный пул повторных размещений раз в месяц. Какую скидку сможете дать на первый тестовый запуск?». В 80% случаев скидывают 15-20%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>Правило 4: Единый UTM-стандарт</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>Для каждого канала строго своя ссылка: https://ai-rop.ru/?utm_source=tg&amp;utm_medium={код_канала}&amp;utm_campaign=audit3. В Яндекс.Метрике (ID: 113329268) сразу отслеживаем стоимость лида (CPL) и конверсию.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="29">
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A32:J32"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="D39:J39"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="A35:J35"/>
+    <mergeCell ref="A38:J38"/>
+    <mergeCell ref="D42:J42"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A31:J31"/>
+    <mergeCell ref="A30:J30"/>
+    <mergeCell ref="A34:J34"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A36:J36"/>
+    <mergeCell ref="D40:J40"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="D41:J41"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A33:J33"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(battlecard): add imot.io competitor battlecard and switch-offer to founder workspace
</commit_message>
<xml_diff>
--- a/docs/RevOps_Founder_Workspace_Planner.xlsx
+++ b/docs/RevOps_Founder_Workspace_Planner.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -178,6 +178,30 @@
       <b val="1"/>
       <color rgb="00059669"/>
       <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00047857"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="12">
@@ -367,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -546,6 +570,30 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1625,7 +1673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1978,10 +2026,248 @@
       <c r="F26" s="38" t="n"/>
       <c r="G26" s="37" t="n"/>
     </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="68" t="inlineStr">
+        <is>
+          <t>⚔️ БАТТЛКАРТА КОНКУРЕНТОВ: REVOPS OS vs IMOT.IO (И ДРУГИЕ ПОМИНУТНЫЕ РЕЧЕВЫЕ АНАЛИТИКИ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="69" t="inlineStr">
+        <is>
+          <t>Анатомия конкурента: ООО «Имотио» (Сколково). Тарифы от 54 000 до 400 000 ₽/мес за пакеты минут. Скрипты перехвата клиентов:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="70" t="inlineStr">
+        <is>
+          <t>Параметр сравнения</t>
+        </is>
+      </c>
+      <c r="B30" s="70" t="inlineStr">
+        <is>
+          <t>Imot.io (Классический ASR/ОКК)</t>
+        </is>
+      </c>
+      <c r="C30" s="70" t="inlineStr">
+        <is>
+          <t>RevOps Enterprise OS PRO (ai-rop.ru)</t>
+        </is>
+      </c>
+      <c r="D30" s="70" t="inlineStr">
+        <is>
+          <t>Решающее преимущество RevOps</t>
+        </is>
+      </c>
+      <c r="E30" s="70" t="inlineStr">
+        <is>
+          <t>Скрипт перехвата клиента</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="71" t="inlineStr">
+        <is>
+          <t>Тарификация и масштабирование</t>
+        </is>
+      </c>
+      <c r="B31" s="71" t="inlineStr">
+        <is>
+          <t>Поминутная (54k – 400k ₽/мес). Чем дольше говорят менеджеры, тем выше счет. Ограничение минут.</t>
+        </is>
+      </c>
+      <c r="C31" s="72" t="inlineStr">
+        <is>
+          <t>Фиксированная цена за модуль с БЕЗЛИМИТОМ минут (от 29k ₽/мес). Ноль переплат за секунды.</t>
+        </is>
+      </c>
+      <c r="D31" s="71" t="inlineStr">
+        <is>
+          <t>Нет «налога на разговоры». 100% диалогов анализируются без страха исчерпать лимит.</t>
+        </is>
+      </c>
+      <c r="E31" s="71" t="inlineStr">
+        <is>
+          <t>«В Imot.io вы платите штраф за то, что продавцы долго общаются с клиентами. В RevOps OS — полный безлимит по честной фикс-цене».</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" s="73" t="inlineStr">
+        <is>
+          <t>Скорость спасения сделки</t>
+        </is>
+      </c>
+      <c r="B32" s="73" t="inlineStr">
+        <is>
+          <t>Постфактум в веб-дашборде через 24–48 часов. РОП должен сам копаться в графиках.</t>
+        </is>
+      </c>
+      <c r="C32" s="74" t="inlineStr">
+        <is>
+          <t>Мгновенный Telegram-алертер за 30 секунд со сценарием спасения сделки прямо в кармане РОПа.</t>
+        </is>
+      </c>
+      <c r="D32" s="73" t="inlineStr">
+        <is>
+          <t>Сделку перехватывают день-в-день, пока клиент не ушел к конкурентам.</t>
+        </is>
+      </c>
+      <c r="E32" s="73" t="inlineStr">
+        <is>
+          <t>«Пока Imot.io рисует графики, наш бот за 30 секунд присылает готовый скрипт, как перехватить уходящую сделку на 500 000 ₽».</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="71" t="inlineStr">
+        <is>
+          <t>Отношение отдела продаж</t>
+        </is>
+      </c>
+      <c r="B33" s="71" t="inlineStr">
+        <is>
+          <t>Инструмент тотальной слежки («Большой Брат»). Саботаж звонков, уход в личный WhatsApp, увольнения.</t>
+        </is>
+      </c>
+      <c r="C33" s="72" t="inlineStr">
+        <is>
+          <t>Пакет «Антисаботаж» и Режим «Адвокат менеджера». ИИ защищает от токсичных клиентов и не штрафует.</t>
+        </is>
+      </c>
+      <c r="D33" s="71" t="inlineStr">
+        <is>
+          <t>Менеджеры любят систему, так как она освобождает 40 мин/день и защищает перед руководством.</t>
+        </is>
+      </c>
+      <c r="E33" s="71" t="inlineStr">
+        <is>
+          <t>«Imot.io внедряется как надзиратель со штрафами. RevOps OS — это адвокат менеджера, который снимает рутину и защищает от несправедливых санкций».</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="73" t="inlineStr">
+        <is>
+          <t>Фокус на деньгах и выручке</t>
+        </is>
+      </c>
+      <c r="B34" s="73" t="inlineStr">
+        <is>
+          <t>Отвлеченные баллы качества речи (7.8/10), стоп-слова, приветствия без привязки к кассе.</t>
+        </is>
+      </c>
+      <c r="C34" s="74" t="inlineStr">
+        <is>
+          <t>Оцифровка денежного риска сделки в рублях (28% речи, 18% КП, 10% DSO). Сквозной ROI.</t>
+        </is>
+      </c>
+      <c r="D34" s="73" t="inlineStr">
+        <is>
+          <t>Разговор с собственником на языке кассы и чистой прибыли, а не скриптов.</t>
+        </is>
+      </c>
+      <c r="E34" s="73" t="inlineStr">
+        <is>
+          <t>«Баллы за скрипт не платят зарплату. Мы оцифровываем конкретный финансовый риск: сколько рублей под угрозой прямо сейчас».</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" s="71" t="inlineStr">
+        <is>
+          <t>Автозаполнение CRM-системы</t>
+        </is>
+      </c>
+      <c r="B35" s="71" t="inlineStr">
+        <is>
+          <t>Требует ручного заполнения полей или передает только базовые теги и расшифровку текста.</t>
+        </is>
+      </c>
+      <c r="C35" s="72" t="inlineStr">
+        <is>
+          <t>Полное автозаполнение CRM: Executive Summary разговора, BANT-потребности и дата Next Step.</t>
+        </is>
+      </c>
+      <c r="D35" s="71" t="inlineStr">
+        <is>
+          <t>Экономия 40 минут рабочего времени каждого продавца в день.</t>
+        </is>
+      </c>
+      <c r="E35" s="71" t="inlineStr">
+        <is>
+          <t>«Ваши продавцы больше не тратят время на заполнение CRM — нейросеть делает это за них идеально».</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" s="73" t="inlineStr">
+        <is>
+          <t>Входной барьер и тест-драйв</t>
+        </is>
+      </c>
+      <c r="B36" s="73" t="inlineStr">
+        <is>
+          <t>Запись на демо через сайт, длинный пресейл, пилот от 50 000 ₽ по договору.</t>
+        </is>
+      </c>
+      <c r="C36" s="74" t="inlineStr">
+        <is>
+          <t>Бесплатный экспресс тест-драйв 3 звонков за 15 минут в Telegram-боте (0 ₽).</t>
+        </is>
+      </c>
+      <c r="D36" s="73" t="inlineStr">
+        <is>
+          <t>Мгновенная демонстрация ценности на реальных звонках клиента до оплаты.</t>
+        </is>
+      </c>
+      <c r="E36" s="73" t="inlineStr">
+        <is>
+          <t>«Загрузите 3 вчерашних звонка в наш Telegram-бот — через 15 минут получите оцифровку риска бесплатно».</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" s="71" t="inlineStr">
+        <is>
+          <t>Оффер миграции (Switch Offer)</t>
+        </is>
+      </c>
+      <c r="B37" s="71" t="inlineStr">
+        <is>
+          <t>Нет программы переезда (продают только свои минуты).</t>
+        </is>
+      </c>
+      <c r="C37" s="72" t="inlineStr">
+        <is>
+          <t>Бесплатный перенос настроек и словарей за 1 день + 1 месяц безлимита в подарок при переходе.</t>
+        </is>
+      </c>
+      <c r="D37" s="71" t="inlineStr">
+        <is>
+          <t>Убийственный крючок для переключения действующих клиентов Imot.io.</t>
+        </is>
+      </c>
+      <c r="E37" s="71" t="inlineStr">
+        <is>
+          <t>«Перенесем ваши настройки из Imot.io за 1 день и подарим первый месяц обслуживания бесплатно».</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="75" t="inlineStr">
+        <is>
+          <t>🎁 ГОТОВЫЙ SWITCH-ОФФЕР ДЛЯ МАРКЕТИНГА: «ПЛАТИТЕ ЗА МИНУТЫ В IMOT.IO? ПЕРЕХОДИТЕ НА БЕЗЛИМИТ REVOPS OS ЗА 1 ДЕНЬ + МЕСЯЦ В ПОДАРОК!»</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="41">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="D18:G18"/>
+    <mergeCell ref="A39:E39"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="A8:G8"/>
     <mergeCell ref="D25:G25"/>
@@ -2014,7 +2300,9 @@
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A29:E29"/>
     <mergeCell ref="D17:G17"/>
+    <mergeCell ref="A28:E28"/>
     <mergeCell ref="D16:G16"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A16:C16"/>
@@ -6799,31 +7087,31 @@
           <t>💰 БЮДЖЕТ ТЕСТА</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n"/>
+      <c r="B4" s="37" t="n"/>
       <c r="C4" s="55" t="inlineStr">
         <is>
           <t>👁️ ЦЕЛЕВОЙ ОХВАТ</t>
         </is>
       </c>
-      <c r="D4" s="25" t="n"/>
+      <c r="D4" s="37" t="n"/>
       <c r="E4" s="54" t="inlineStr">
         <is>
           <t>🎯 КЛИКИ НА САЙТ (CTR ~2.5%)</t>
         </is>
       </c>
-      <c r="F4" s="25" t="n"/>
+      <c r="F4" s="37" t="n"/>
       <c r="G4" s="56" t="inlineStr">
         <is>
           <t>📥 ЗАЯВКИ НА АУДИТ (0 ₽)</t>
         </is>
       </c>
-      <c r="H4" s="25" t="n"/>
+      <c r="H4" s="37" t="n"/>
       <c r="I4" s="57" t="inlineStr">
         <is>
           <t>🚀 ЗАКРЫТЫЕ ПИЛОТЫ (ROI)</t>
         </is>
       </c>
-      <c r="J4" s="25" t="n"/>
+      <c r="J4" s="37" t="n"/>
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="58" t="inlineStr">
@@ -6831,31 +7119,31 @@
           <t>35 000 – 60 000 ₽</t>
         </is>
       </c>
-      <c r="B5" s="25" t="n"/>
+      <c r="B5" s="37" t="n"/>
       <c r="C5" s="59" t="inlineStr">
         <is>
           <t>15 000 – 35 000 Views</t>
         </is>
       </c>
-      <c r="D5" s="25" t="n"/>
+      <c r="D5" s="37" t="n"/>
       <c r="E5" s="60" t="inlineStr">
         <is>
           <t>450 – 850 кликов</t>
         </is>
       </c>
-      <c r="F5" s="25" t="n"/>
+      <c r="F5" s="37" t="n"/>
       <c r="G5" s="61" t="inlineStr">
         <is>
           <t>25 – 45 заявок</t>
         </is>
       </c>
-      <c r="H5" s="25" t="n"/>
+      <c r="H5" s="37" t="n"/>
       <c r="I5" s="62" t="inlineStr">
         <is>
           <t>3 – 6 сделок (165к-360к ₽)</t>
         </is>
       </c>
-      <c r="J5" s="25" t="n"/>
+      <c r="J5" s="37" t="n"/>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
@@ -7969,6 +8257,15 @@
           <t>📌 Пост 1 (Комбо: Продажи + CRM) | Для каналов: @crm50, @completo_ru, @Salesnotes, @crm_secrets, @introvert_crm</t>
         </is>
       </c>
+      <c r="B31" s="38" t="n"/>
+      <c r="C31" s="38" t="n"/>
+      <c r="D31" s="38" t="n"/>
+      <c r="E31" s="38" t="n"/>
+      <c r="F31" s="38" t="n"/>
+      <c r="G31" s="38" t="n"/>
+      <c r="H31" s="38" t="n"/>
+      <c r="I31" s="38" t="n"/>
+      <c r="J31" s="37" t="n"/>
     </row>
     <row r="32" ht="110" customHeight="1">
       <c r="A32" s="31" t="inlineStr">
@@ -7988,6 +8285,15 @@
 👉 [Получить экспресс-аудит 3 звонков (0 ₽)] {ССЫЛКА_С_UTM}</t>
         </is>
       </c>
+      <c r="B32" s="38" t="n"/>
+      <c r="C32" s="38" t="n"/>
+      <c r="D32" s="38" t="n"/>
+      <c r="E32" s="38" t="n"/>
+      <c r="F32" s="38" t="n"/>
+      <c r="G32" s="38" t="n"/>
+      <c r="H32" s="38" t="n"/>
+      <c r="I32" s="38" t="n"/>
+      <c r="J32" s="37" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="67" t="inlineStr">
@@ -7995,6 +8301,15 @@
           <t>📌 Пост 2 (Кейс-разбор в стиле шоу Гребенюка) | Для каналов: @resulting_ru, @biz_razbory, @floor_99, @batyrev_maxim, @grafsky_b2b</t>
         </is>
       </c>
+      <c r="B33" s="38" t="n"/>
+      <c r="C33" s="38" t="n"/>
+      <c r="D33" s="38" t="n"/>
+      <c r="E33" s="38" t="n"/>
+      <c r="F33" s="38" t="n"/>
+      <c r="G33" s="38" t="n"/>
+      <c r="H33" s="38" t="n"/>
+      <c r="I33" s="38" t="n"/>
+      <c r="J33" s="37" t="n"/>
     </row>
     <row r="34" ht="110" customHeight="1">
       <c r="A34" s="31" t="inlineStr">
@@ -8014,6 +8329,15 @@
 👉 [Проверить 3 звонка отдела продаж (0 ₽)] {ССЫЛКА_С_UTM}</t>
         </is>
       </c>
+      <c r="B34" s="38" t="n"/>
+      <c r="C34" s="38" t="n"/>
+      <c r="D34" s="38" t="n"/>
+      <c r="E34" s="38" t="n"/>
+      <c r="F34" s="38" t="n"/>
+      <c r="G34" s="38" t="n"/>
+      <c r="H34" s="38" t="n"/>
+      <c r="I34" s="38" t="n"/>
+      <c r="J34" s="37" t="n"/>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="67" t="inlineStr">
@@ -8021,6 +8345,15 @@
           <t>📌 Пост 3 (Переманивание клиентов с imot.io и Mango) | Для каналов: @rocketsales_blog, @introvert_crm, @ai_business_ru, @crm50</t>
         </is>
       </c>
+      <c r="B35" s="38" t="n"/>
+      <c r="C35" s="38" t="n"/>
+      <c r="D35" s="38" t="n"/>
+      <c r="E35" s="38" t="n"/>
+      <c r="F35" s="38" t="n"/>
+      <c r="G35" s="38" t="n"/>
+      <c r="H35" s="38" t="n"/>
+      <c r="I35" s="38" t="n"/>
+      <c r="J35" s="37" t="n"/>
     </row>
     <row r="36" ht="110" customHeight="1">
       <c r="A36" s="31" t="inlineStr">
@@ -8036,6 +8369,15 @@
 👉 [Узнать условия переезда и получить тест 3 звонков] {ССЫЛКА_С_UTM}</t>
         </is>
       </c>
+      <c r="B36" s="38" t="n"/>
+      <c r="C36" s="38" t="n"/>
+      <c r="D36" s="38" t="n"/>
+      <c r="E36" s="38" t="n"/>
+      <c r="F36" s="38" t="n"/>
+      <c r="G36" s="38" t="n"/>
+      <c r="H36" s="38" t="n"/>
+      <c r="I36" s="38" t="n"/>
+      <c r="J36" s="37" t="n"/>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
@@ -8050,11 +8392,19 @@
           <t>Правило 1: Проверка через TGStat</t>
         </is>
       </c>
+      <c r="B39" s="38" t="n"/>
+      <c r="C39" s="37" t="n"/>
       <c r="D39" s="16" t="inlineStr">
         <is>
           <t>Перед оплатой обязательно вбейте канал на tgstat.ru. Смотрите на ER (вовлеченность должна быть &gt;15-20%) и график суточного охвата: если посты читают равномерно, а не скачком в 03:00 ночи — накрутки ботами нет.</t>
         </is>
       </c>
+      <c r="E39" s="38" t="n"/>
+      <c r="F39" s="38" t="n"/>
+      <c r="G39" s="38" t="n"/>
+      <c r="H39" s="38" t="n"/>
+      <c r="I39" s="38" t="n"/>
+      <c r="J39" s="37" t="n"/>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="14" t="inlineStr">
@@ -8062,11 +8412,19 @@
           <t>Правило 2: Формат размещения 2/48</t>
         </is>
       </c>
+      <c r="B40" s="38" t="n"/>
+      <c r="C40" s="37" t="n"/>
       <c r="D40" s="16" t="inlineStr">
         <is>
           <t>Не берите 1/24 (быстро смоется лентой). Для длинных экспертных постов B2B просите формат 2/48 (2 часа в топе без перекрытия другими постами и 48 часов в ленте), либо формат 'без удаления'.</t>
         </is>
       </c>
+      <c r="E40" s="38" t="n"/>
+      <c r="F40" s="38" t="n"/>
+      <c r="G40" s="38" t="n"/>
+      <c r="H40" s="38" t="n"/>
+      <c r="I40" s="38" t="n"/>
+      <c r="J40" s="37" t="n"/>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="14" t="inlineStr">
@@ -8074,11 +8432,19 @@
           <t>Правило 3: Скрипт торга со скидкой 10-20%</t>
         </is>
       </c>
+      <c r="B41" s="38" t="n"/>
+      <c r="C41" s="37" t="n"/>
       <c r="D41" s="16" t="inlineStr">
         <is>
           <t>Пишите админу прямо: «Тестируем новый ИИ-сервис для B2B отделов продаж. Если отдача будет хорошей — зайдем на постоянный пул повторных размещений раз в месяц. Какую скидку сможете дать на первый тестовый запуск?». В 80% случаев скидывают 15-20%.</t>
         </is>
       </c>
+      <c r="E41" s="38" t="n"/>
+      <c r="F41" s="38" t="n"/>
+      <c r="G41" s="38" t="n"/>
+      <c r="H41" s="38" t="n"/>
+      <c r="I41" s="38" t="n"/>
+      <c r="J41" s="37" t="n"/>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
@@ -8086,11 +8452,19 @@
           <t>Правило 4: Единый UTM-стандарт</t>
         </is>
       </c>
+      <c r="B42" s="38" t="n"/>
+      <c r="C42" s="37" t="n"/>
       <c r="D42" s="16" t="inlineStr">
         <is>
           <t>Для каждого канала строго своя ссылка: https://ai-rop.ru/?utm_source=tg&amp;utm_medium={код_канала}&amp;utm_campaign=audit3. В Яндекс.Метрике (ID: 113329268) сразу отслеживаем стоимость лида (CPL) и конверсию.</t>
         </is>
       </c>
+      <c r="E42" s="38" t="n"/>
+      <c r="F42" s="38" t="n"/>
+      <c r="G42" s="38" t="n"/>
+      <c r="H42" s="38" t="n"/>
+      <c r="I42" s="38" t="n"/>
+      <c r="J42" s="37" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="29">

</xml_diff>